<commit_message>
Append trimika data — 16 new rows, 31 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1745,6 +1745,1358 @@
       <c r="Q16" t="inlineStr">
         <is>
           <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2565606</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EF4-0231310-2</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2026-04-22 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2565607</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>EF4-0231311-0</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2026-04-22 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2565774</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>EF4-0231546-1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>VA923704988</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-06-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2026-05-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2565609</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>EF4-0231681-6</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>VA923704988</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1076</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>PREMET</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>172704-21182</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>2026-04-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2565750</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>EF4-0231718-6</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>V0710315396</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>9803.00.50</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>SUBSTANTIAL CONTAINERS US&amp;INTL</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>9803.00.50</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>MEBROM LLC</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>MEBLLC01</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>84-463527000</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>SAHAMITR PRESSURE CONTAINER PUBLIC</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SAHAMITR PRESSURE CONTAINER PUBLIC CO LTD</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>2026-05-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2565714</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>EF4-0231746-7</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>V1P06243667</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1108.14.0000</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2565716</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>EF4-0231748-3</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>V1P06243667</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1108.14.0000</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2565715</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EF4-0232019-8</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>V1P06243667</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1108.14.0000</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2565725</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EF4-0232228-5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>V1P06243667</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>9903.82.09,8302.42.3015</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>GRASS AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>GRAAME</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>51-066023000</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>GRASS GMBH</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>GRASS GMBH</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>2026-05-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2566081</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>EF4-0232237-6</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.40.9000</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>IMS GEAR VIRGINIA LLC</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>IMSGEA</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>20-800570900</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2566081</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>EF4-0232237-6</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.40.9000</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>IMS GEAR VIRGINIA LLC</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>IMSGEA</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>20-800570900</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2566081</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>EF4-0232237-6</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.40.9000</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>IMS GEAR VIRGINIA LLC</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>IMSGEA</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>20-800570900</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2566081</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>EF4-0232237-6</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.40.9000</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>IMS GEAR VIRGINIA LLC</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>IMSGEA</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>20-800570900</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2566081</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>EF4-0232237-6</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.40.9000</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>IMS GEAR VIRGINIA LLC</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>IMSGEA</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>20-800570900</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2566081</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>EF4-0232237-6</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.40.9000</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>IMS GEAR VIRGINIA LLC</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>IMSGEA</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>20-800570900</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>ADOLF FOHL GMBH &amp; CO.</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>4539450</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>EF4-0232402-6</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>9903.90.08,2931.90.9052</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>EREZTECH LLC</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ERELLC01</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>27-437122900</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>SYNOR LTD</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SYNOR LTD</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append trimika data — 34 new rows, 65 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3100,6 +3100,2828 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>5402.61.0000</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>5402.61.0000</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>5402.61.0000</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>5606.00.0010</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>5402.62.0000</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>5402.52.9000</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>5402.33.3000</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>5402.33.3000</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>5402.61.0000</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>5402.61.0000</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>5402.52.9000</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>5402.51.0000</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>5402.61.0000</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2565646</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>EF4-0231408-4</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>5606.00.0010</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HICKORY THROWING COMPANY</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>HICTHR</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>56-124106800</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SARLA PERFORMANCE FIBERS LTD</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2565772</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>EF4-0231545-3</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>5603.14.9090</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2565681</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>EF4-0231551-1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>V0710311346</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>5603.14.9090</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-06-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2565767</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>EF4-0231554-5</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>V0710311346</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>5603.14.9090</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2565717</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>EF4-0231634-5</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>1108.14.0000</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>SOUTHEAST ASIA ORGANIC CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>SOUTHEAST ASIA ORGANIC CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>105504693</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>EF4-0231692-3</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>2026-05-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>105504694</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>EF4-0231694-9</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>2026-05-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>105504702</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>EF4-0231794-7</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>2026-05-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>105504703</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EF4-0231801-0</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>2026-05-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>105504718</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>EF4-0231836-6</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>105504719</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>EF4-0231837-4</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>2026-05-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2565843</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>EF4-0231944-8</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIAC</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIACZANEGO PEPEES S.A.</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>2026-05-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2565900</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>EF4-0232029-7</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>9903.82.10,8428.33.0000</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>AUMUND CORPORATION</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>AUMCOR</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>58-138896800</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>2026-05-18 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2565816</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>EF4-0232058-6</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>1109.00.9010</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>2026-05-22 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2565857</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>EF4-0232060-2</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>2026-05-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2566034</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>EF4-0232180-8</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>V1626455557</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>1108.11.0010</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2566053</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>EF4-0232278-0</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>V1626455557</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2566053</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EF4-0232278-0</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>V1626455557</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2566053</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>EF4-0232278-0</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>V1626455557</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2566053</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>EF4-0232278-0</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>V1626455557</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2566053</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>EF4-0232278-0</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>V1626455557</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 36 new rows, 101 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q66"/>
+  <dimension ref="A1:Q102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5922,6 +5922,3026 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2565494</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>EF4-0231250-0</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>ROQUETTE FRERES</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>ROQUETTE FRERES</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>2026-04-18 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2565534</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>EF4-0231273-2</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>2026-04-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2565697</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>EF4-0231423-3</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>2026-04-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2565660</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>EF4-0231430-8</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>2026-04-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2565924</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>EF4-0231960-4</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>2026-05-18 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2566052</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>EF4-0232193-1</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>3402.90.1000</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>SCHILL SEILACHER GMBH CO</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>SCHILL SEILACHER GMBH CO</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2566057</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>EF4-0232211-1</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>V1626460482</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2566058</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>EF4-0232213-7</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>V1626460482</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2566067</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>EF4-0232214-5</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>V1626460482</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2566070</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>EF4-0232215-2</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>V1626460482</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>4539358</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>EF4-0232235-0</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>01650618422</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>3204.19.2020</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>COLORCHEM INTERNATIONAL CORP</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>COLORC01</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>58-241511400</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>PHILODEN INDUSTRIES PVT LTD</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>PHILODEN INDUSTRIES PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2566145</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>EF4-0232245-9</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>01650618422</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>1109.00.9010</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>FILTERTECHNIK EUROPE GMBH &amp; CO KG</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>FILTERTECHNIK EUROPE GMBH &amp; CO KG</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>WIREMESH-PRO TEC GMBH</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>WIREMESH-PRO TEC GMBH</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>WIREMESH-PRO TEC GMBH</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>WIREMESH-PRO TEC GMBH</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>WIREMESH-PRO TEC GMBH</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>WIREMESH-PRO TEC GMBH</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>8448.20.5090</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>3402.90.5030</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>8421.99.0180</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>5911.32.0080</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>8477.90.8695</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>REIFENHAUSER REICOFIL GMBH &amp; CO. KG</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>8448.32.0090</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>HASTEM GMBH</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>HASTEM GMBH</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>8448.32.0090</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>HASTEM GMBH</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>HASTEM GMBH</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>8453.90.5000</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>BRUCKNER AFTER SALES GMBH</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>BRUCKNER AFTER SALES GMBH</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>8516.10.0080</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>BRUCKNER AFTER SALES GMBH</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>BRUCKNER AFTER SALES GMBH</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>3403.99.0000</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>BRUCKNER AFTER SALES GMBH</t>
+        </is>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>BRUCKNER AFTER SALES GMBH</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>8448.39.9000</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>ZENTES UNITEX GMBH</t>
+        </is>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>ZENTES UNITEX GMBH</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>4811.49.3000</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>ZENTES UNITEX GMBH</t>
+        </is>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>ZENTES UNITEX GMBH</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2566233</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EF4-0232259-0</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>4811.49.3000</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>FI-TECH INC</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>FITINC</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>54-091465000</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>ZENTES UNITEX GMBH</t>
+        </is>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>ZENTES UNITEX GMBH</t>
+        </is>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2565794</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>EF4-0232384-6</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>V0413916151</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1031</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
+        </is>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2566107</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>EF4-0232386-1</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>V0413916151</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>5503.40.0000</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>FOOTING FIRST, LLC</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>FOOFIR</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>27-059921300</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>HAGELSON PLASTIK GERI DONUSUM VE NA</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>HAGELSON PLASTIK GERI DONUSUM VE NAKLIYE SANAYI TICARET ANONIM SIRKETI</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>4539413</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>EF4-0232400-0</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>3405.20.0000</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>COVE HOME LLC</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>COVHOM01</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>30-136116600</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>CV. PRASDA BALI UTMA</t>
+        </is>
+      </c>
+      <c r="P100" t="inlineStr">
+        <is>
+          <t>CV. PRASDA BALI UTMA</t>
+        </is>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>4539413</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>EF4-0232400-0</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>4419.20.9000</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>COVE HOME LLC</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>COVHOM01</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>30-136116600</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>CV. PRASDA BALI UTMA</t>
+        </is>
+      </c>
+      <c r="P101" t="inlineStr">
+        <is>
+          <t>CV. PRASDA BALI UTMA</t>
+        </is>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>4539413</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>EF4-0232400-0</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>4202.22.1500</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>COVE HOME LLC</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>COVHOM01</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>30-136116600</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>CV. PRASDA BALI UTMA</t>
+        </is>
+      </c>
+      <c r="P102" t="inlineStr">
+        <is>
+          <t>CV. PRASDA BALI UTMA</t>
+        </is>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 20 new rows, 121 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q102"/>
+  <dimension ref="A1:Q122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8942,6 +8942,1638 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2565751</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>EF4-0231790-5</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>9903.82.10,8428.33.0000</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>AUMUND CORPORATION</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>AUMCOR</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>58-138896800</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="P103" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>2026-05-11 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2565927</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EF4-0231897-8</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>3920.62.0090</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>GULF ATLANTIC PACKAGING CORP</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>GULATL</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>58-184378700</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>CONSENT FZCO</t>
+        </is>
+      </c>
+      <c r="P104" t="inlineStr">
+        <is>
+          <t>CONSENT FZCO</t>
+        </is>
+      </c>
+      <c r="Q104" t="inlineStr">
+        <is>
+          <t>2026-05-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2566010</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>EF4-0231962-0</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIAC</t>
+        </is>
+      </c>
+      <c r="P105" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIACZANEGO PEPEES S.A.</t>
+        </is>
+      </c>
+      <c r="Q105" t="inlineStr">
+        <is>
+          <t>2026-05-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2565855</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>EF4-0232059-4</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>V1626451887</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P106" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q106" t="inlineStr">
+        <is>
+          <t>2026-05-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2566011</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>EF4-0232062-8</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>V1626451887</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIAC</t>
+        </is>
+      </c>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIACZANEGO PEPEES S.A.</t>
+        </is>
+      </c>
+      <c r="Q107" t="inlineStr">
+        <is>
+          <t>2026-05-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2566028</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>EF4-0232065-1</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>V0710334942</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>1108.12.0010</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>2026-05-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>105504734</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>EF4-0232081-8</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>105504735</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>EF4-0232084-2</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P110" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q110" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>105504736</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>EF4-0232087-5</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2565712</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>EF4-0232088-3</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>9903.82.09,9403.20.0075</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P112" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q112" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2565712</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>EF4-0232088-3</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>9903.76.04,9403.60.8093</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q113" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2565712</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>EF4-0232088-3</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P114" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q114" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2565712</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>EF4-0232088-3</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>VIET MOI INDUSTRIAL COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>105504738</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>EF4-0232095-8</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P116" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>105504739</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>EF4-0232096-6</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P117" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q117" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>105504740</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>EF4-0232098-2</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>105504741</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>EF4-0232100-6</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>2026-05-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>105504747</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>EF4-0232107-1</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P120" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q120" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2566131</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>EF4-0232126-1</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>V1626459831</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>1108.12.0010</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="P121" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="Q121" t="inlineStr">
+        <is>
+          <t>2026-05-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2565958</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>EF4-0232210-3</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>V1626459831</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>BORGERS OHIO INC.</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>BORUSA02</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>30-084196200</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 28 new rows, 163 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q137"/>
+  <dimension ref="A1:Q164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9889,12 +9889,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2565958</t>
+          <t>2565664</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EF4-0232210-3</t>
+          <t>EF4-0231432-4</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -9902,19 +9902,15 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>V1626459831</t>
-        </is>
-      </c>
+      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -9924,64 +9920,64 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+          <t>5903.90.3090</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>BORGERS OHIO INC.</t>
+          <t>VEER CORPORATIONS INC</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>BORUSA02</t>
+          <t>VEECOR01</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>30-084196200</t>
+          <t>99-106989200</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>2026-06-15 00:00:00</t>
+          <t>2026-06-14 00:00:00</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>2026-06-13 00:00:00</t>
+          <t>2026-06-14 00:00:00</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>VEER PLASTIC PVT LTD</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>VEER PLASTIC PVT LTD</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>2026-05-28 00:00:00</t>
+          <t>2026-04-27 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2565664</t>
+          <t>2565647</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>EF4-0231432-4</t>
+          <t>EF4-0231683-2</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -10012,47 +10008,47 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>5903.90.3090</t>
+          <t>3305.10.0000</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>VEER CORPORATIONS INC</t>
+          <t>ETHIQUE CONSUMER PRODUCTS, INC</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>VEECOR01</t>
+          <t>ETHCO01</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>99-106989200</t>
+          <t>85-417193400</t>
         </is>
       </c>
       <c r="M116" t="inlineStr">
         <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
           <t>2026-06-14 00:00:00</t>
         </is>
       </c>
-      <c r="N116" t="inlineStr">
-        <is>
-          <t>2026-06-14 00:00:00</t>
-        </is>
-      </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>VEER PLASTIC PVT LTD</t>
+          <t>SHIELING LABORATORIES LTD</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>VEER PLASTIC PVT LTD</t>
+          <t>SHIELING LABORATORIES LTD</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>2026-04-27 00:00:00</t>
+          <t>2026-05-05 00:00:00</t>
         </is>
       </c>
     </row>
@@ -10085,7 +10081,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -10095,7 +10091,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>3305.10.0000</t>
+          <t>3305.90.0000</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -10168,7 +10164,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -10178,7 +10174,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>3305.90.0000</t>
+          <t>3307.20.0000</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -10251,7 +10247,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -10261,7 +10257,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>3307.20.0000</t>
+          <t>3305.10.0000</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -10308,12 +10304,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2565647</t>
+          <t>2565873</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EF4-0231683-2</t>
+          <t>EF4-0231852-3</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -10334,7 +10330,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -10344,22 +10340,22 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>3305.10.0000</t>
+          <t>9903.82.01,8431.20.0000</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>ETHIQUE CONSUMER PRODUCTS, INC</t>
+          <t>MALLAGHAN (GA) INC.</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>ETHCO01</t>
+          <t>MALGA01</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>85-417193400</t>
+          <t>36-488102800</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
@@ -10374,29 +10370,29 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>SHIELING LABORATORIES LTD</t>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>SHIELING LABORATORIES LTD</t>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>2026-05-05 00:00:00</t>
+          <t>2026-05-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2565873</t>
+          <t>2565888</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EF4-0231852-3</t>
+          <t>EF4-0231959-6</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -10404,7 +10400,11 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>V0710337820</t>
+        </is>
+      </c>
       <c r="E121" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -10427,27 +10427,27 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>9903.82.01,8431.20.0000</t>
+          <t>1108.13.0010</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>MALLAGHAN (GA) INC.</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>MALGA01</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>36-488102800</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>2026-06-15 00:00:00</t>
+          <t>2026-06-14 00:00:00</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -10457,29 +10457,29 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>MALLAGHAN ENGINEERING  LTD</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>MALLAGHAN ENGINEERING  LTD</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>2026-05-12 00:00:00</t>
+          <t>2026-05-18 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2565888</t>
+          <t>2565945</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EF4-0231959-6</t>
+          <t>EF4-0231961-2</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -10497,11 +10497,7 @@
           <t>9903.03.01</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>SECTION 122 - 10% DUTY</t>
-        </is>
-      </c>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>001</t>
@@ -10534,57 +10530,61 @@
       </c>
       <c r="M122" t="inlineStr">
         <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
           <t>2026-06-14 00:00:00</t>
         </is>
       </c>
-      <c r="N122" t="inlineStr">
-        <is>
-          <t>2026-06-14 00:00:00</t>
-        </is>
-      </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIAC</t>
         </is>
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIACZANEGO PEPEES S.A.</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>2026-05-18 00:00:00</t>
+          <t>2026-05-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2565945</t>
+          <t>2615692</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EF4-0231961-2</t>
+          <t>EF4-0231982-8</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
+          <t>Vessel, Non-container</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>V0710337820</t>
+          <t>V8N03137232</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr"/>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
       <c r="G123" t="inlineStr">
         <is>
           <t>001</t>
@@ -10592,32 +10592,32 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>1108.13.0010</t>
+          <t>9903.03.01,3926.90.9989</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>BORGERS OHIO INC.</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>BORUSA02</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>30-084196200</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
         <is>
-          <t>2026-06-15 00:00:00</t>
+          <t>2026-06-04 00:00:00</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -10627,17 +10627,17 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIAC</t>
+          <t>AUTONEUM (SHANGHAI) MANAGEMENT CO.</t>
         </is>
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIACZANEGO PEPEES S.A.</t>
+          <t>AUTONEUM (SHANGHAI) MANAGEMENT CO. LTD.</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>2026-05-17 00:00:00</t>
+          <t>2026-05-19 00:00:00</t>
         </is>
       </c>
     </row>
@@ -10674,7 +10674,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -10684,7 +10684,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>9903.03.01,3926.90.9989</t>
+          <t>9903.03.01,3926.30.5000</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -10731,17 +10731,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2615692</t>
+          <t>2565999</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EF4-0231982-8</t>
+          <t>EF4-0232009-9</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Vessel, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10751,47 +10751,47 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>9903.03.01,3926.30.5000</t>
+          <t>1806.90.9090</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>BORGERS OHIO INC.</t>
+          <t>DOBLA USA MFG LLC</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>BORUSA02</t>
+          <t>DOBUSA</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>30-084196200</t>
+          <t>41-218954800</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>2026-06-04 00:00:00</t>
+          <t>2026-06-15 00:00:00</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -10801,12 +10801,12 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>AUTONEUM (SHANGHAI) MANAGEMENT CO.</t>
+          <t>DOBLA LOGISTICS BVBA</t>
         </is>
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>AUTONEUM (SHANGHAI) MANAGEMENT CO. LTD.</t>
+          <t>DOBLA LOGISTICS BVBA</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -10818,12 +10818,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2565999</t>
+          <t>2565956</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>EF4-0232009-9</t>
+          <t>EF4-0232032-1</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -10831,11 +10831,7 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>V8N03137232</t>
-        </is>
-      </c>
+      <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -10858,22 +10854,22 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>1806.90.9090</t>
+          <t>9903.82.01,8431.20.0000</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>MALLAGHAN (GA) INC.</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>MALGA01</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>36-488102800</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
@@ -10888,12 +10884,12 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>DOBLA LOGISTICS BVBA</t>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
         </is>
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>DOBLA LOGISTICS BVBA</t>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -10905,12 +10901,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2565956</t>
+          <t>2566028</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>EF4-0232032-1</t>
+          <t>EF4-0232065-1</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -10924,11 +10920,7 @@
           <t>9903.03.01</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>SECTION 122 - 10% DUTY</t>
-        </is>
-      </c>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>001</t>
@@ -10941,27 +10933,27 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>9903.82.01,8431.20.0000</t>
+          <t>1108.12.0010</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>MALLAGHAN (GA) INC.</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>MALGA01</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>36-488102800</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>2026-06-15 00:00:00</t>
+          <t>2026-06-14 00:00:00</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -10971,29 +10963,29 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>MALLAGHAN ENGINEERING  LTD</t>
+          <t>TAT NISASTA INS SAN TIC AS</t>
         </is>
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>MALLAGHAN ENGINEERING  LTD</t>
+          <t>TAT NISASTA INS SAN TIC AS</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>2026-05-19 00:00:00</t>
+          <t>2026-05-23 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2566028</t>
+          <t>2566055</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>EF4-0232065-1</t>
+          <t>EF4-0232124-6</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -11001,13 +10993,21 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>V0710343679</t>
+        </is>
+      </c>
       <c r="E128" t="inlineStr">
         <is>
           <t>9903.03.01</t>
         </is>
       </c>
-      <c r="F128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
       <c r="G128" t="inlineStr">
         <is>
           <t>001</t>
@@ -11020,7 +11020,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>1108.12.0010</t>
+          <t>1109.00.9020</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -11050,29 +11050,29 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>TAT NISASTA INS SAN TIC AS</t>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>TAT NISASTA INS SAN TIC AS</t>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>2026-05-23 00:00:00</t>
+          <t>2026-05-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2566055</t>
+          <t>2566131</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EF4-0232124-6</t>
+          <t>EF4-0232126-1</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -11090,11 +11090,7 @@
           <t>9903.03.01</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>SECTION 122 - 10% DUTY</t>
-        </is>
-      </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>001</t>
@@ -11107,7 +11103,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>1109.00.9020</t>
+          <t>1108.12.0010</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -11137,29 +11133,29 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+          <t>TAT NISASTA INS SAN TIC AS</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+          <t>TAT NISASTA INS SAN TIC AS</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>2026-05-25 00:00:00</t>
+          <t>2026-05-23 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2566131</t>
+          <t>2566056</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>EF4-0232126-1</t>
+          <t>EF4-0232208-7</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -11169,7 +11165,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>V0710343679</t>
+          <t>V1626459831</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -11177,7 +11173,11 @@
           <t>9903.03.01</t>
         </is>
       </c>
-      <c r="F130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
       <c r="G130" t="inlineStr">
         <is>
           <t>001</t>
@@ -11190,7 +11190,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>1108.12.0010</t>
+          <t>1108.13.0010</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -11220,29 +11220,29 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>TAT NISASTA INS SAN TIC AS</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>TAT NISASTA INS SAN TIC AS</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>2026-05-23 00:00:00</t>
+          <t>2026-05-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2566056</t>
+          <t>2566180</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EF4-0232208-7</t>
+          <t>EF4-0232260-8</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -11250,11 +11250,7 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>V1626459831</t>
-        </is>
-      </c>
+      <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -11277,59 +11273,59 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>1108.13.0010</t>
+          <t>9903.82.01,8424.90.9080</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>EISINC03</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>86-240963300</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
         <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
           <t>2026-06-14 00:00:00</t>
         </is>
       </c>
-      <c r="N131" t="inlineStr">
-        <is>
-          <t>2026-06-14 00:00:00</t>
-        </is>
-      </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>EISENMANN GMBH</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>EISENMANN GMBH</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>2026-05-25 00:00:00</t>
+          <t>2026-06-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2566180</t>
+          <t>2566053</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EF4-0232260-8</t>
+          <t>EF4-0232278-0</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -11340,12 +11336,12 @@
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -11355,27 +11351,27 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>9903.82.01,8424.90.9080</t>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>EISINC03</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>86-240963300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
@@ -11390,12 +11386,12 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>EISENMANN GMBH</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>EISENMANN GMBH</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
@@ -11433,7 +11429,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -11516,7 +11512,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -11599,7 +11595,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -11682,7 +11678,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>005</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -11739,12 +11735,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2566053</t>
+          <t>2565851</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EF4-0232278-0</t>
+          <t>EF4-0231710-3</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -11752,70 +11748,2403 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>VA923744786</t>
+        </is>
+      </c>
       <c r="E137" t="inlineStr">
         <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>2026-05-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2565884</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>EF4-0231856-4</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>VA923744786</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2930.90.9231</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>CASTLE CHEMICALS LTD</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>CASCHE01</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>151704-07138</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>2026-05-13 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2565885</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>EF4-0231857-2</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2930.90.9231</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>CASTLE CHEMICALS LTD</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>CASCHE01</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>151704-07138</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>2026-05-13 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2565886</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>EF4-0231858-0</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2930.90.9231</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>CASTLE CHEMICALS LTD</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>CASCHE01</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>151704-07138</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>2026-05-13 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2565875</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>EF4-0231949-7</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2931.49.0055</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>BRUHL CHEMICAL TRADE INC</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>BRUCHE02</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>83-155181000</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>HUBEI GURUN TECHNOLOGY CO. LTD</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>HUBEI GURUN TECHNOLOGY CO. LTD</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>2026-05-13 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2565860</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>EF4-0232030-5</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr">
+        <is>
           <t>9903.03.06</t>
         </is>
       </c>
-      <c r="F137" t="inlineStr">
+      <c r="F142" t="inlineStr">
         <is>
           <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr">
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>9903.82.10,8415.81.0130</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>SUNBELT RENTALS, INC.</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>SUNREN01</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>58-041519200</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>HEPHZIBAH CO LTD</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>HEPHZIBAH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>2026-05-21 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2565860</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>EF4-0232030-5</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>9903.82.10,8415.81.0130</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>SUNBELT RENTALS, INC.</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>SUNREN01</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>58-041519200</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>HEPHZIBAH CO LTD</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>HEPHZIBAH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>2026-05-21 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2566066</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>EF4-0232182-4</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>V1626459823</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>1702.30.4085</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>2026-06-16 00:00:00</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>AK NISASTA SANAYI VE TICARET AS</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>AK NISASTA SANAYI VE TICARET AS</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2565958</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>EF4-0232210-3</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>V1626459823</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>BORGERS OHIO INC.</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>BORUSA02</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>30-084196200</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>8481.80.9050</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>9903.82.10,8479.89.9599</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>8501.31.2000</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>9903.82.02,7320.90.5060</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
         <is>
           <t>005</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr">
+      <c r="H150" t="inlineStr">
         <is>
           <t>9903.03.06</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
-        <is>
-          <t>9903.74.11,9903.94.53,8708.29.5160</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>BORGERS USA CORP</t>
-        </is>
-      </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>BORUSA</t>
-        </is>
-      </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>65-117296500</t>
-        </is>
-      </c>
-      <c r="M137" t="inlineStr">
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>9903.82.02,7320.90.5060</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
         <is>
           <t>2026-06-12 00:00:00</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr">
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
         <is>
           <t>2026-06-14 00:00:00</t>
         </is>
       </c>
-      <c r="O137" t="inlineStr">
-        <is>
-          <t>AUTONEUM CZ S.R.O.</t>
-        </is>
-      </c>
-      <c r="P137" t="inlineStr">
-        <is>
-          <t>AUTONEUM CZ S.R.O.</t>
-        </is>
-      </c>
-      <c r="Q137" t="inlineStr">
-        <is>
-          <t>2026-06-01 00:00:00</t>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>8414.59.6595</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>9903.82.02,7320.90.5060</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>9903.94.06,8537.10.9160</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>4016.93.5050</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>8481.80.9050</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>8504.40.9540</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>9903.82.09,8302.10.6090</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>4539483</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>EF4-0232485-1</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>V9S19229198</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>8443.91.3000</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>EUROPEAN SPARE PARTS SERVICE INC</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>ESSEUR</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>58-181585100</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>2026-06-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>HJK INTERNATIONAL GMBH</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append trimika data — 21 new rows, 305 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q285"/>
+  <dimension ref="A1:Q306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24227,6 +24227,1781 @@
         </is>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2565718</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>EF4-0231703-8</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr"/>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>3505.10.0092</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>EHM INTERTRADING CO LTD</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>EHM INTERTRADING CO LTD</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>2026-05-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2565827</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>EF4-0231709-5</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr"/>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>2026-05-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr"/>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr"/>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr"/>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr"/>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr"/>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr"/>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2565938</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>EF4-0231958-8</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr"/>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2615664</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>EF4-0231983-6</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr"/>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>9903.88.01</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(A)</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>9903.88.01</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8482.10.5012</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>LINYU HANDWARE MANUFACTURE CO LTD</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>LINYU HANDWARE MANUFACTURE CO LTD</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>2026-05-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2565682</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>EF4-0231989-3</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr"/>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>9903.03.01,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2565682</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>EF4-0231989-3</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr"/>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>9903.03.01,9405.41.8440</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2565682</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>EF4-0231989-3</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr"/>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2565800</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>EF4-0232068-5</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>V0413939047</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1031</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>2026-05-11 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2566097</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>EF4-0232212-9</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>V0413939047</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>5704.90.0190</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>BORGERS OHIO INC.</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>BORUSA02</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>30-084196200</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>AUTONEUM GERMANY GMBH</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>AUTONEUM GERMANY GMBH</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2566097</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>EF4-0232212-9</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>V0413939047</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>5704.90.0190</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>BORGERS OHIO INC.</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>BORUSA02</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>30-084196200</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>AUTONEUM GERMANY GMBH</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>AUTONEUM GERMANY GMBH</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2566097</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>EF4-0232212-9</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>V0413939047</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>5704.90.0190</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>BORGERS OHIO INC.</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>BORUSA02</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>30-084196200</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>AUTONEUM GERMANY GMBH</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>AUTONEUM GERMANY GMBH</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2565838</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>EF4-0232439-8</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>V0413931663</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0062</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2565907</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>EF4-0232496-8</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>V0413937900</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0043</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>2026-05-11 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2565907</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>EF4-0232496-8</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>V0413937900</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0073</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>2026-05-11 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2615809</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>EF4-0232557-7</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Truck, Non-container</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>V0413937900</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>8483.40.5010</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>AUMUND CORPORATION</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>AUMCOR</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>58-138896800</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>2026-06-16 00:00:00</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>2026-06-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 17 new rows, 322 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q306"/>
+  <dimension ref="A1:Q323"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26002,6 +26002,1417 @@
         </is>
       </c>
     </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2565634</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>EF4-0231631-1</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr"/>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>8438.90.9060</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>CANTRELL GAINCO GROUP INC</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>CANGAI01</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>31-151121700</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2565782</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>EF4-0231677-4</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr"/>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>3505.10.0092</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>EHM INTERTRADING CO LTD</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>EHM INTERTRADING CO LTD</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2565784</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>EF4-0231678-2</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr"/>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>3505.10.0092</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>EHM INTERTRADING CO LTD</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>EHM INTERTRADING CO LTD</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2565894</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>EF4-0232004-0</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr"/>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>2930.90.9231</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>CASTLE CHEMICALS LTD</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>CASCHE01</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>151704-07138</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>2026-04-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2566078</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>EF4-0232219-4</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr"/>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>8474.10.0010</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>EDGE INNOVATE (NI) LTD</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>EDGINN01</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>135501-01432</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>EDGE INNOVATE (NI) LTD</t>
+        </is>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>EDGE INNOVATE (NI) LTD</t>
+        </is>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>2026-05-29 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2565937</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>EF4-0232258-2</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr"/>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>9903.82.22,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>2026-05-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2565937</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>EF4-0232258-2</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr"/>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>9903.82.22,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P313" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>2026-05-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2565937</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>EF4-0232258-2</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr"/>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>9903.82.22,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N314" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P314" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>2026-05-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2566105</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>EF4-0232283-0</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr"/>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>3920.61.0000</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>TUBUS BAUER GMBH</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>TUBBAU01</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>091601-00584</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>TUBUS BAUER GMBH</t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>TUBUS BAUER GMBH</t>
+        </is>
+      </c>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2566265</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>EF4-0232362-2</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr"/>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>9903.82.01,8424.90.9080</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N316" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2566155</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>EF4-0232431-5</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2566155</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>EF4-0232431-5</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr"/>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N318" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q318" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2566155</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>EF4-0232431-5</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr"/>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2566155</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>EF4-0232431-5</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr"/>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q320" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>4539433</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>EF4-0232434-9</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr"/>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>9903.03.03,2926.90.4300</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>MAYZO INC</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>MAYINC</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>62-129031200</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>HANGZHOU DISHENG IMPORT &amp; EXPORT</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>HANGZHOU DISHENG IMPORT &amp; EXPORT</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2565798</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>EF4-0232494-3</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr"/>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0064</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N322" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2565799</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>EF4-0232495-0</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr"/>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0062</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 18 new rows, 339 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q323"/>
+  <dimension ref="A1:Q340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24977,28 +24977,28 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>2615664</t>
+          <t>2565682</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>EF4-0231983-6</t>
+          <t>EF4-0231989-3</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Vessel, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D295" t="inlineStr"/>
       <c r="E295" t="inlineStr">
         <is>
-          <t>9903.88.01</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(A)</t>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -25008,12 +25008,12 @@
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>9903.88.01</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>9903.03.06,9903.82.09,8482.10.5012</t>
+          <t>9903.03.01,9403.99.9045</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
@@ -25033,7 +25033,7 @@
       </c>
       <c r="M295" t="inlineStr">
         <is>
-          <t>2026-06-11 00:00:00</t>
+          <t>2026-06-19 00:00:00</t>
         </is>
       </c>
       <c r="N295" t="inlineStr">
@@ -25043,17 +25043,17 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>LINYU HANDWARE MANUFACTURE CO LTD</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>LINYU HANDWARE MANUFACTURE CO LTD</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr">
         <is>
-          <t>2026-05-15 00:00:00</t>
+          <t>2026-05-19 00:00:00</t>
         </is>
       </c>
     </row>
@@ -25086,7 +25086,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -25096,7 +25096,7 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>9903.03.01,9403.99.9045</t>
+          <t>9903.03.01,9405.41.8440</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
@@ -25159,27 +25159,27 @@
       <c r="D297" t="inlineStr"/>
       <c r="E297" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>9903.03.01,9405.41.8440</t>
+          <t>9903.03.01,3926.90.9989</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
@@ -25226,12 +25226,12 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>2565682</t>
+          <t>2565800</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>EF4-0231989-3</t>
+          <t>EF4-0232068-5</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -25239,50 +25239,54 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D298" t="inlineStr"/>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>V0413939047</t>
+        </is>
+      </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>9903.03.01,3926.90.9989</t>
+          <t>9903.82.02,7223.00.1031</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
         <is>
-          <t>VISUAL CREATIONS, INC.</t>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
         <is>
-          <t>VISCRE</t>
+          <t>VENWIR</t>
         </is>
       </c>
       <c r="L298" t="inlineStr">
         <is>
-          <t>20-461602300</t>
+          <t>993901-03595</t>
         </is>
       </c>
       <c r="M298" t="inlineStr">
         <is>
-          <t>2026-06-19 00:00:00</t>
+          <t>2026-06-17 00:00:00</t>
         </is>
       </c>
       <c r="N298" t="inlineStr">
@@ -25292,29 +25296,29 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
         </is>
       </c>
       <c r="Q298" t="inlineStr">
         <is>
-          <t>2026-05-19 00:00:00</t>
+          <t>2026-05-11 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>2565800</t>
+          <t>2566097</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>EF4-0232068-5</t>
+          <t>EF4-0232212-9</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -25329,12 +25333,12 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
@@ -25344,27 +25348,27 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>9903.82.02,7223.00.1031</t>
+          <t>5704.90.0190</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+          <t>BORGERS OHIO INC.</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
         <is>
-          <t>VENWIR</t>
+          <t>BORUSA02</t>
         </is>
       </c>
       <c r="L299" t="inlineStr">
         <is>
-          <t>993901-03595</t>
+          <t>30-084196200</t>
         </is>
       </c>
       <c r="M299" t="inlineStr">
@@ -25379,17 +25383,17 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
+          <t>AUTONEUM GERMANY GMBH</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
+          <t>AUTONEUM GERMANY GMBH</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr">
         <is>
-          <t>2026-05-11 00:00:00</t>
+          <t>2026-05-30 00:00:00</t>
         </is>
       </c>
     </row>
@@ -25426,7 +25430,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
@@ -25513,7 +25517,7 @@
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
@@ -25570,12 +25574,12 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>2566097</t>
+          <t>2565838</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>EF4-0232212-9</t>
+          <t>EF4-0232439-8</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -25585,47 +25589,47 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>V0413939047</t>
+          <t>V0413931663</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>5704.90.0190</t>
+          <t>9903.82.02,7222.20.0062</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>BORGERS OHIO INC.</t>
+          <t>MESHA STEELS  LLC</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
         <is>
-          <t>BORUSA02</t>
+          <t>MESSTE</t>
         </is>
       </c>
       <c r="L302" t="inlineStr">
         <is>
-          <t>30-084196200</t>
+          <t>20-274801900</t>
         </is>
       </c>
       <c r="M302" t="inlineStr">
@@ -25640,29 +25644,29 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>AUTONEUM GERMANY GMBH</t>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
         </is>
       </c>
       <c r="P302" t="inlineStr">
         <is>
-          <t>AUTONEUM GERMANY GMBH</t>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
         </is>
       </c>
       <c r="Q302" t="inlineStr">
         <is>
-          <t>2026-05-30 00:00:00</t>
+          <t>2026-05-05 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>2565838</t>
+          <t>2565907</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>EF4-0232439-8</t>
+          <t>EF4-0232496-8</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -25672,7 +25676,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>V0413931663</t>
+          <t>V0413937900</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
@@ -25697,7 +25701,7 @@
       </c>
       <c r="I303" t="inlineStr">
         <is>
-          <t>9903.82.02,7222.20.0062</t>
+          <t>9903.82.02,7222.20.0043</t>
         </is>
       </c>
       <c r="J303" t="inlineStr">
@@ -25737,7 +25741,7 @@
       </c>
       <c r="Q303" t="inlineStr">
         <is>
-          <t>2026-05-05 00:00:00</t>
+          <t>2026-05-11 00:00:00</t>
         </is>
       </c>
     </row>
@@ -25774,7 +25778,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
@@ -25784,7 +25788,7 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>9903.82.02,7222.20.0043</t>
+          <t>9903.82.02,7222.20.0073</t>
         </is>
       </c>
       <c r="J304" t="inlineStr">
@@ -25831,17 +25835,17 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>2565907</t>
+          <t>2615809</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>EF4-0232496-8</t>
+          <t>EF4-0232557-7</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
+          <t>Truck, Non-container</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
@@ -25851,91 +25855,87 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
         <is>
-          <t>9903.82.02,7222.20.0073</t>
+          <t>8483.40.5010</t>
         </is>
       </c>
       <c r="J305" t="inlineStr">
         <is>
-          <t>MESHA STEELS  LLC</t>
+          <t>AUMUND CORPORATION</t>
         </is>
       </c>
       <c r="K305" t="inlineStr">
         <is>
-          <t>MESSTE</t>
+          <t>AUMCOR</t>
         </is>
       </c>
       <c r="L305" t="inlineStr">
         <is>
-          <t>20-274801900</t>
+          <t>58-138896800</t>
         </is>
       </c>
       <c r="M305" t="inlineStr">
         <is>
+          <t>2026-06-16 00:00:00</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
           <t>2026-06-17 00:00:00</t>
         </is>
       </c>
-      <c r="N305" t="inlineStr">
-        <is>
-          <t>2026-06-17 00:00:00</t>
-        </is>
-      </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
         </is>
       </c>
       <c r="P305" t="inlineStr">
         <is>
-          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
         </is>
       </c>
       <c r="Q305" t="inlineStr">
         <is>
-          <t>2026-05-11 00:00:00</t>
+          <t>2026-06-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>2615809</t>
+          <t>2565634</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>EF4-0232557-7</t>
+          <t>EF4-0231631-1</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Truck, Non-container</t>
-        </is>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>V0413937900</t>
-        </is>
-      </c>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr"/>
       <c r="E306" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -25958,59 +25958,59 @@
       </c>
       <c r="I306" t="inlineStr">
         <is>
-          <t>8483.40.5010</t>
+          <t>8438.90.9060</t>
         </is>
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>AUMUND CORPORATION</t>
+          <t>CANTRELL GAINCO GROUP INC</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
         <is>
-          <t>AUMCOR</t>
+          <t>CANGAI01</t>
         </is>
       </c>
       <c r="L306" t="inlineStr">
         <is>
-          <t>58-138896800</t>
+          <t>31-151121700</t>
         </is>
       </c>
       <c r="M306" t="inlineStr">
         <is>
-          <t>2026-06-16 00:00:00</t>
+          <t>2026-06-18 00:00:00</t>
         </is>
       </c>
       <c r="N306" t="inlineStr">
         <is>
-          <t>2026-06-17 00:00:00</t>
+          <t>2026-06-18 00:00:00</t>
         </is>
       </c>
       <c r="O306" t="inlineStr">
         <is>
-          <t>AUMUND FOERDERTECHNIK GMBH</t>
+          <t>O E CO LTD</t>
         </is>
       </c>
       <c r="P306" t="inlineStr">
         <is>
-          <t>AUMUND FOERDERTECHNIK GMBH</t>
+          <t>O E CO LTD</t>
         </is>
       </c>
       <c r="Q306" t="inlineStr">
         <is>
-          <t>2026-06-16 00:00:00</t>
+          <t>2026-05-05 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>2565634</t>
+          <t>2565782</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>EF4-0231631-1</t>
+          <t>EF4-0231677-4</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -26041,22 +26041,22 @@
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>8438.90.9060</t>
+          <t>3505.10.0092</t>
         </is>
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>CANTRELL GAINCO GROUP INC</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
         <is>
-          <t>CANGAI01</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L307" t="inlineStr">
         <is>
-          <t>31-151121700</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M307" t="inlineStr">
@@ -26071,12 +26071,12 @@
       </c>
       <c r="O307" t="inlineStr">
         <is>
-          <t>O E CO LTD</t>
+          <t>EHM INTERTRADING CO LTD</t>
         </is>
       </c>
       <c r="P307" t="inlineStr">
         <is>
-          <t>O E CO LTD</t>
+          <t>EHM INTERTRADING CO LTD</t>
         </is>
       </c>
       <c r="Q307" t="inlineStr">
@@ -26088,12 +26088,12 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>2565782</t>
+          <t>2565784</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>EF4-0231677-4</t>
+          <t>EF4-0231678-2</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -26171,12 +26171,12 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>2565784</t>
+          <t>2565894</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>EF4-0231678-2</t>
+          <t>EF4-0232004-0</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -26187,12 +26187,12 @@
       <c r="D309" t="inlineStr"/>
       <c r="E309" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.03</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
@@ -26202,27 +26202,27 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.03</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
-          <t>3505.10.0092</t>
+          <t>2930.90.9231</t>
         </is>
       </c>
       <c r="J309" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>CASTLE CHEMICALS LTD</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>CASCHE01</t>
         </is>
       </c>
       <c r="L309" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>151704-07138</t>
         </is>
       </c>
       <c r="M309" t="inlineStr">
@@ -26237,45 +26237,45 @@
       </c>
       <c r="O309" t="inlineStr">
         <is>
-          <t>EHM INTERTRADING CO LTD</t>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
         </is>
       </c>
       <c r="P309" t="inlineStr">
         <is>
-          <t>EHM INTERTRADING CO LTD</t>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
         </is>
       </c>
       <c r="Q309" t="inlineStr">
         <is>
-          <t>2026-05-05 00:00:00</t>
+          <t>2026-04-30 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>2565894</t>
+          <t>2566078</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>EF4-0232004-0</t>
+          <t>EF4-0232219-4</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
+          <t>Vessel, Non-container</t>
         </is>
       </c>
       <c r="D310" t="inlineStr"/>
       <c r="E310" t="inlineStr">
         <is>
-          <t>9903.03.03</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
@@ -26285,80 +26285,80 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>9903.03.03</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
         <is>
-          <t>2930.90.9231</t>
+          <t>8474.10.0010</t>
         </is>
       </c>
       <c r="J310" t="inlineStr">
         <is>
-          <t>CASTLE CHEMICALS LTD</t>
+          <t>EDGE INNOVATE (NI) LTD</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
         <is>
-          <t>CASCHE01</t>
+          <t>EDGINN01</t>
         </is>
       </c>
       <c r="L310" t="inlineStr">
         <is>
-          <t>151704-07138</t>
+          <t>135501-01432</t>
         </is>
       </c>
       <c r="M310" t="inlineStr">
         <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
           <t>2026-06-18 00:00:00</t>
         </is>
       </c>
-      <c r="N310" t="inlineStr">
-        <is>
-          <t>2026-06-18 00:00:00</t>
-        </is>
-      </c>
       <c r="O310" t="inlineStr">
         <is>
-          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
+          <t>EDGE INNOVATE (NI) LTD</t>
         </is>
       </c>
       <c r="P310" t="inlineStr">
         <is>
-          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
+          <t>EDGE INNOVATE (NI) LTD</t>
         </is>
       </c>
       <c r="Q310" t="inlineStr">
         <is>
-          <t>2026-04-30 00:00:00</t>
+          <t>2026-05-29 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>2566078</t>
+          <t>2565937</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>EF4-0232219-4</t>
+          <t>EF4-0232258-2</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Vessel, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D311" t="inlineStr"/>
       <c r="E311" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
@@ -26368,32 +26368,32 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
         <is>
-          <t>8474.10.0010</t>
+          <t>9903.82.22,8431.20.0000</t>
         </is>
       </c>
       <c r="J311" t="inlineStr">
         <is>
-          <t>EDGE INNOVATE (NI) LTD</t>
+          <t>MALLAGHAN (GA) INC.</t>
         </is>
       </c>
       <c r="K311" t="inlineStr">
         <is>
-          <t>EDGINN01</t>
+          <t>MALGA01</t>
         </is>
       </c>
       <c r="L311" t="inlineStr">
         <is>
-          <t>135501-01432</t>
+          <t>36-488102800</t>
         </is>
       </c>
       <c r="M311" t="inlineStr">
         <is>
-          <t>2026-06-17 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
       <c r="N311" t="inlineStr">
@@ -26403,17 +26403,17 @@
       </c>
       <c r="O311" t="inlineStr">
         <is>
-          <t>EDGE INNOVATE (NI) LTD</t>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
         </is>
       </c>
       <c r="P311" t="inlineStr">
         <is>
-          <t>EDGE INNOVATE (NI) LTD</t>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
         </is>
       </c>
       <c r="Q311" t="inlineStr">
         <is>
-          <t>2026-05-29 00:00:00</t>
+          <t>2026-05-17 00:00:00</t>
         </is>
       </c>
     </row>
@@ -26446,7 +26446,7 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
@@ -26529,7 +26529,7 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
@@ -26586,12 +26586,12 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>2565937</t>
+          <t>2566105</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>EF4-0232258-2</t>
+          <t>EF4-0232283-0</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -26602,47 +26602,47 @@
       <c r="D314" t="inlineStr"/>
       <c r="E314" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
         <is>
-          <t>9903.82.22,8431.20.0000</t>
+          <t>3920.61.0000</t>
         </is>
       </c>
       <c r="J314" t="inlineStr">
         <is>
-          <t>MALLAGHAN (GA) INC.</t>
+          <t>TUBUS BAUER GMBH</t>
         </is>
       </c>
       <c r="K314" t="inlineStr">
         <is>
-          <t>MALGA01</t>
+          <t>TUBBAU01</t>
         </is>
       </c>
       <c r="L314" t="inlineStr">
         <is>
-          <t>36-488102800</t>
+          <t>091601-00584</t>
         </is>
       </c>
       <c r="M314" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-18 00:00:00</t>
         </is>
       </c>
       <c r="N314" t="inlineStr">
@@ -26652,29 +26652,29 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>MALLAGHAN ENGINEERING  LTD</t>
+          <t>TUBUS BAUER GMBH</t>
         </is>
       </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>MALLAGHAN ENGINEERING  LTD</t>
+          <t>TUBUS BAUER GMBH</t>
         </is>
       </c>
       <c r="Q314" t="inlineStr">
         <is>
-          <t>2026-05-17 00:00:00</t>
+          <t>2026-06-02 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>2566105</t>
+          <t>2566265</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>EF4-0232283-0</t>
+          <t>EF4-0232362-2</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -26705,59 +26705,59 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>3920.61.0000</t>
+          <t>9903.82.01,8424.90.9080</t>
         </is>
       </c>
       <c r="J315" t="inlineStr">
         <is>
-          <t>TUBUS BAUER GMBH</t>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
         <is>
-          <t>TUBBAU01</t>
+          <t>EISINC03</t>
         </is>
       </c>
       <c r="L315" t="inlineStr">
         <is>
-          <t>091601-00584</t>
+          <t>86-240963300</t>
         </is>
       </c>
       <c r="M315" t="inlineStr">
         <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr">
+        <is>
           <t>2026-06-18 00:00:00</t>
         </is>
       </c>
-      <c r="N315" t="inlineStr">
-        <is>
-          <t>2026-06-18 00:00:00</t>
-        </is>
-      </c>
       <c r="O315" t="inlineStr">
         <is>
-          <t>TUBUS BAUER GMBH</t>
+          <t>EISENMANN GMBH</t>
         </is>
       </c>
       <c r="P315" t="inlineStr">
         <is>
-          <t>TUBUS BAUER GMBH</t>
+          <t>EISENMANN GMBH</t>
         </is>
       </c>
       <c r="Q315" t="inlineStr">
         <is>
-          <t>2026-06-02 00:00:00</t>
+          <t>2026-06-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>2566265</t>
+          <t>2566155</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>EF4-0232362-2</t>
+          <t>EF4-0232431-5</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -26768,12 +26768,12 @@
       <c r="D316" t="inlineStr"/>
       <c r="E316" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -26783,32 +26783,32 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
         <is>
-          <t>9903.82.01,8424.90.9080</t>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
         </is>
       </c>
       <c r="J316" t="inlineStr">
         <is>
-          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
         <is>
-          <t>EISINC03</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L316" t="inlineStr">
         <is>
-          <t>86-240963300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M316" t="inlineStr">
         <is>
-          <t>2026-06-21 00:00:00</t>
+          <t>2026-06-18 00:00:00</t>
         </is>
       </c>
       <c r="N316" t="inlineStr">
@@ -26818,12 +26818,12 @@
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t>EISENMANN GMBH</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P316" t="inlineStr">
         <is>
-          <t>EISENMANN GMBH</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q316" t="inlineStr">
@@ -26861,7 +26861,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
@@ -26944,7 +26944,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
@@ -27027,7 +27027,7 @@
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
@@ -27084,111 +27084,111 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>2566155</t>
+          <t>4539433</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>EF4-0232431-5</t>
+          <t>EF4-0232434-9</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
+          <t>Air, Non-container</t>
         </is>
       </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+          <t>9903.03.03,2926.90.4300</t>
         </is>
       </c>
       <c r="J320" t="inlineStr">
         <is>
-          <t>BORGERS USA CORP</t>
+          <t>MAYZO INC</t>
         </is>
       </c>
       <c r="K320" t="inlineStr">
         <is>
-          <t>BORUSA</t>
+          <t>MAYINC</t>
         </is>
       </c>
       <c r="L320" t="inlineStr">
         <is>
-          <t>65-117296500</t>
+          <t>62-129031200</t>
         </is>
       </c>
       <c r="M320" t="inlineStr">
         <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr">
+        <is>
           <t>2026-06-18 00:00:00</t>
         </is>
       </c>
-      <c r="N320" t="inlineStr">
-        <is>
-          <t>2026-06-18 00:00:00</t>
-        </is>
-      </c>
       <c r="O320" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>HANGZHOU DISHENG IMPORT &amp; EXPORT</t>
         </is>
       </c>
       <c r="P320" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>HANGZHOU DISHENG IMPORT &amp; EXPORT</t>
         </is>
       </c>
       <c r="Q320" t="inlineStr">
         <is>
-          <t>2026-06-06 00:00:00</t>
+          <t>2026-06-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>4539433</t>
+          <t>2565798</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>EF4-0232434-9</t>
+          <t>EF4-0232494-3</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
@@ -27198,32 +27198,32 @@
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>9903.03.03,2926.90.4300</t>
+          <t>9903.82.02,7222.20.0064</t>
         </is>
       </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>MAYZO INC</t>
+          <t>MESHA STEELS  LLC</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
         <is>
-          <t>MAYINC</t>
+          <t>MESSTE</t>
         </is>
       </c>
       <c r="L321" t="inlineStr">
         <is>
-          <t>62-129031200</t>
+          <t>20-274801900</t>
         </is>
       </c>
       <c r="M321" t="inlineStr">
         <is>
-          <t>2026-06-17 00:00:00</t>
+          <t>2026-06-18 00:00:00</t>
         </is>
       </c>
       <c r="N321" t="inlineStr">
@@ -27233,29 +27233,29 @@
       </c>
       <c r="O321" t="inlineStr">
         <is>
-          <t>HANGZHOU DISHENG IMPORT &amp; EXPORT</t>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
         </is>
       </c>
       <c r="P321" t="inlineStr">
         <is>
-          <t>HANGZHOU DISHENG IMPORT &amp; EXPORT</t>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
         </is>
       </c>
       <c r="Q321" t="inlineStr">
         <is>
-          <t>2026-06-17 00:00:00</t>
+          <t>2026-05-12 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2565798</t>
+          <t>2565799</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>EF4-0232494-3</t>
+          <t>EF4-0232495-0</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -27286,7 +27286,7 @@
       </c>
       <c r="I322" t="inlineStr">
         <is>
-          <t>9903.82.02,7222.20.0064</t>
+          <t>9903.82.02,7222.20.0062</t>
         </is>
       </c>
       <c r="J322" t="inlineStr">
@@ -27333,12 +27333,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>2565799</t>
+          <t>2565760</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>EF4-0232495-0</t>
+          <t>EF4-0231661-8</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -27349,67 +27349,1498 @@
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8302.42.3015</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>GRASS AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>GRAAME</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>51-066023000</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>SACA PRECISION LTD</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>SACA PRECISION LTD</t>
+        </is>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2565760</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>EF4-0231661-8</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr"/>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.30.5000</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>GRASS AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>GRAAME</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>51-066023000</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N324" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>SACA PRECISION LTD</t>
+        </is>
+      </c>
+      <c r="P324" t="inlineStr">
+        <is>
+          <t>SACA PRECISION LTD</t>
+        </is>
+      </c>
+      <c r="Q324" t="inlineStr">
+        <is>
+          <t>2026-05-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2615656</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>EF4-0231976-0</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr"/>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N325" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>NINGBO SMART HIGH TECH INDUSTRIES L</t>
+        </is>
+      </c>
+      <c r="P325" t="inlineStr">
+        <is>
+          <t>NINGBO SMART HIGH TECH INDUSTRIES LTD</t>
+        </is>
+      </c>
+      <c r="Q325" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2615664</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>EF4-0231983-6</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr"/>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>9903.88.01</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(A)</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>9903.88.01</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8482.10.5012</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N326" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>LINYU HANDWARE MANUFACTURE CO LTD</t>
+        </is>
+      </c>
+      <c r="P326" t="inlineStr">
+        <is>
+          <t>LINYU HANDWARE MANUFACTURE CO LTD</t>
+        </is>
+      </c>
+      <c r="Q326" t="inlineStr">
+        <is>
+          <t>2026-05-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2565923</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>EF4-0232195-6</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr"/>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>9903.91.01</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>ARTS, PRDS OF CN SUB(B)US NT31</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>9903.91.01</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.02,7228.30.6000</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>MAHA USA LLC</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>MAHUSA</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>52-213556300</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N327" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="P327" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="Q327" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2565923</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>EF4-0232195-6</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr"/>
+      <c r="E328" t="inlineStr">
+        <is>
           <t>9903.03.06</t>
         </is>
       </c>
-      <c r="F323" t="inlineStr">
+      <c r="F328" t="inlineStr">
         <is>
           <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
-      <c r="G323" t="inlineStr">
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>9903.82.02,7215.50.0016</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>MAHA USA LLC</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>MAHUSA</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>52-213556300</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N328" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="P328" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="Q328" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2565923</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>EF4-0232195-6</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr"/>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>9903.82.02,7216.33.0090</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>MAHA USA LLC</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>MAHUSA</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>52-213556300</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N329" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="P329" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="Q329" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2566178</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>EF4-0232247-5</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr"/>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="H323" t="inlineStr">
-        <is>
-          <t>9903.03.06</t>
-        </is>
-      </c>
-      <c r="I323" t="inlineStr">
-        <is>
-          <t>9903.82.02,7222.20.0062</t>
-        </is>
-      </c>
-      <c r="J323" t="inlineStr">
-        <is>
-          <t>MESHA STEELS  LLC</t>
-        </is>
-      </c>
-      <c r="K323" t="inlineStr">
-        <is>
-          <t>MESSTE</t>
-        </is>
-      </c>
-      <c r="L323" t="inlineStr">
-        <is>
-          <t>20-274801900</t>
-        </is>
-      </c>
-      <c r="M323" t="inlineStr">
-        <is>
-          <t>2026-06-18 00:00:00</t>
-        </is>
-      </c>
-      <c r="N323" t="inlineStr">
-        <is>
-          <t>2026-06-18 00:00:00</t>
-        </is>
-      </c>
-      <c r="O323" t="inlineStr">
-        <is>
-          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
-        </is>
-      </c>
-      <c r="P323" t="inlineStr">
-        <is>
-          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
-        </is>
-      </c>
-      <c r="Q323" t="inlineStr">
-        <is>
-          <t>2026-05-12 00:00:00</t>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N330" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q330" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2566229</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>EF4-0232249-1</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>V0710338448</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N331" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P331" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q331" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2566177</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>EF4-0232275-6</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>V0710338448</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N332" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P332" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q332" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2566051</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>EF4-0232281-4</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>V0710349973</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N333" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q333" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2566051</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>EF4-0232281-4</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>V0710349973</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N334" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q334" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2566051</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>EF4-0232281-4</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>V0710349973</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N335" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O335" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P335" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q335" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2566100</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>EF4-0232282-2</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr"/>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N336" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O336" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P336" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q336" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2566100</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>EF4-0232282-2</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr"/>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N337" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O337" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P337" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q337" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2566100</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>EF4-0232282-2</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr"/>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N338" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O338" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P338" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q338" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2615771</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>EF4-0232406-7</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr"/>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>8210.00.0000</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>COVE HOME LLC</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>COVHOM01</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>30-136116600</t>
+        </is>
+      </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N339" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O339" t="inlineStr">
+        <is>
+          <t>P. IONNOU G ZARKADIS QE</t>
+        </is>
+      </c>
+      <c r="P339" t="inlineStr">
+        <is>
+          <t>P. IONNOU G ZARKADIS QE</t>
+        </is>
+      </c>
+      <c r="Q339" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2615771</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>EF4-0232406-7</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr"/>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>8210.00.0000</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>COVE HOME LLC</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>COVHOM01</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>30-136116600</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N340" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="O340" t="inlineStr">
+        <is>
+          <t>P. IONNOU G ZARKADIS QE</t>
+        </is>
+      </c>
+      <c r="P340" t="inlineStr">
+        <is>
+          <t>P. IONNOU G ZARKADIS QE</t>
+        </is>
+      </c>
+      <c r="Q340" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append trimika data — 16 new rows, 352 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q340"/>
+  <dimension ref="A1:Q353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27665,12 +27665,12 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>2565923</t>
+          <t>2566178</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>EF4-0232195-6</t>
+          <t>EF4-0232247-5</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -27681,12 +27681,12 @@
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr">
         <is>
-          <t>9903.91.01</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>ARTS, PRDS OF CN SUB(B)US NT31</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -27696,27 +27696,27 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>9903.91.01</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I327" t="inlineStr">
         <is>
-          <t>9903.03.06,9903.82.02,7228.30.6000</t>
+          <t>1108.13.0010</t>
         </is>
       </c>
       <c r="J327" t="inlineStr">
         <is>
-          <t>MAHA USA LLC</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K327" t="inlineStr">
         <is>
-          <t>MAHUSA</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L327" t="inlineStr">
         <is>
-          <t>52-213556300</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M327" t="inlineStr">
@@ -27731,29 +27731,29 @@
       </c>
       <c r="O327" t="inlineStr">
         <is>
-          <t>THYSSENKRUPP SCHULTE GMBH</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t>THYSSENKRUPP SCHULTE GMBH</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="Q327" t="inlineStr">
         <is>
-          <t>2026-05-27 00:00:00</t>
+          <t>2026-06-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>2565923</t>
+          <t>2566229</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>EF4-0232195-6</t>
+          <t>EF4-0232249-1</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -27761,45 +27761,49 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr"/>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>V0710338448</t>
+        </is>
+      </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
         <is>
-          <t>9903.82.02,7215.50.0016</t>
+          <t>1108.13.0010</t>
         </is>
       </c>
       <c r="J328" t="inlineStr">
         <is>
-          <t>MAHA USA LLC</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K328" t="inlineStr">
         <is>
-          <t>MAHUSA</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L328" t="inlineStr">
         <is>
-          <t>52-213556300</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M328" t="inlineStr">
@@ -27814,29 +27818,29 @@
       </c>
       <c r="O328" t="inlineStr">
         <is>
-          <t>THYSSENKRUPP SCHULTE GMBH</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="P328" t="inlineStr">
         <is>
-          <t>THYSSENKRUPP SCHULTE GMBH</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="Q328" t="inlineStr">
         <is>
-          <t>2026-05-27 00:00:00</t>
+          <t>2026-06-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>2565923</t>
+          <t>2566177</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>EF4-0232195-6</t>
+          <t>EF4-0232275-6</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -27844,45 +27848,49 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D329" t="inlineStr"/>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>V0710338448</t>
+        </is>
+      </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>9903.82.02,7216.33.0090</t>
+          <t>1108.13.0010</t>
         </is>
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>MAHA USA LLC</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
         <is>
-          <t>MAHUSA</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L329" t="inlineStr">
         <is>
-          <t>52-213556300</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M329" t="inlineStr">
@@ -27897,29 +27905,29 @@
       </c>
       <c r="O329" t="inlineStr">
         <is>
-          <t>THYSSENKRUPP SCHULTE GMBH</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>THYSSENKRUPP SCHULTE GMBH</t>
+          <t>AKV LANGHOLT AMBA</t>
         </is>
       </c>
       <c r="Q329" t="inlineStr">
         <is>
-          <t>2026-05-27 00:00:00</t>
+          <t>2026-06-01 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>2566178</t>
+          <t>2566051</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>EF4-0232247-5</t>
+          <t>EF4-0232281-4</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -27927,7 +27935,11 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D330" t="inlineStr"/>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>V0710349973</t>
+        </is>
+      </c>
       <c r="E330" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -27950,42 +27962,42 @@
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>1108.13.0010</t>
+          <t>4811.59.4040</t>
         </is>
       </c>
       <c r="J330" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
         </is>
       </c>
       <c r="K330" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>BAULIN</t>
         </is>
       </c>
       <c r="L330" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>56-193913400</t>
         </is>
       </c>
       <c r="M330" t="inlineStr">
         <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N330" t="inlineStr">
+        <is>
           <t>2026-06-20 00:00:00</t>
         </is>
       </c>
-      <c r="N330" t="inlineStr">
-        <is>
-          <t>2026-06-20 00:00:00</t>
-        </is>
-      </c>
       <c r="O330" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>SURTECO GMBH</t>
         </is>
       </c>
       <c r="P330" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>SURTECO GMBH</t>
         </is>
       </c>
       <c r="Q330" t="inlineStr">
@@ -27997,12 +28009,12 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>2566229</t>
+          <t>2566051</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>EF4-0232249-1</t>
+          <t>EF4-0232281-4</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -28012,7 +28024,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>V0710338448</t>
+          <t>V0710349973</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -28027,7 +28039,7 @@
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H331" t="inlineStr">
@@ -28037,42 +28049,42 @@
       </c>
       <c r="I331" t="inlineStr">
         <is>
-          <t>1108.13.0010</t>
+          <t>4811.59.4040</t>
         </is>
       </c>
       <c r="J331" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
         </is>
       </c>
       <c r="K331" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>BAULIN</t>
         </is>
       </c>
       <c r="L331" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>56-193913400</t>
         </is>
       </c>
       <c r="M331" t="inlineStr">
         <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N331" t="inlineStr">
+        <is>
           <t>2026-06-20 00:00:00</t>
         </is>
       </c>
-      <c r="N331" t="inlineStr">
-        <is>
-          <t>2026-06-20 00:00:00</t>
-        </is>
-      </c>
       <c r="O331" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>SURTECO GMBH</t>
         </is>
       </c>
       <c r="P331" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>SURTECO GMBH</t>
         </is>
       </c>
       <c r="Q331" t="inlineStr">
@@ -28084,12 +28096,12 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>2566177</t>
+          <t>2566051</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>EF4-0232275-6</t>
+          <t>EF4-0232281-4</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -28099,7 +28111,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>V0710338448</t>
+          <t>V0710349973</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -28114,7 +28126,7 @@
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H332" t="inlineStr">
@@ -28124,42 +28136,42 @@
       </c>
       <c r="I332" t="inlineStr">
         <is>
-          <t>1108.13.0010</t>
+          <t>4811.59.4040</t>
         </is>
       </c>
       <c r="J332" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
         </is>
       </c>
       <c r="K332" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>BAULIN</t>
         </is>
       </c>
       <c r="L332" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>56-193913400</t>
         </is>
       </c>
       <c r="M332" t="inlineStr">
         <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N332" t="inlineStr">
+        <is>
           <t>2026-06-20 00:00:00</t>
         </is>
       </c>
-      <c r="N332" t="inlineStr">
-        <is>
-          <t>2026-06-20 00:00:00</t>
-        </is>
-      </c>
       <c r="O332" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>SURTECO GMBH</t>
         </is>
       </c>
       <c r="P332" t="inlineStr">
         <is>
-          <t>AKV LANGHOLT AMBA</t>
+          <t>SURTECO GMBH</t>
         </is>
       </c>
       <c r="Q332" t="inlineStr">
@@ -28171,12 +28183,12 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>2566051</t>
+          <t>2566100</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>EF4-0232281-4</t>
+          <t>EF4-0232282-2</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -28184,11 +28196,7 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>V0710349973</t>
-        </is>
-      </c>
+      <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -28258,12 +28266,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>2566051</t>
+          <t>2566100</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>EF4-0232281-4</t>
+          <t>EF4-0232282-2</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -28271,11 +28279,7 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr">
-        <is>
-          <t>V0710349973</t>
-        </is>
-      </c>
+      <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -28345,12 +28349,12 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>2566051</t>
+          <t>2566100</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>EF4-0232281-4</t>
+          <t>EF4-0232282-2</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -28358,11 +28362,7 @@
           <t>Vessel, Container</t>
         </is>
       </c>
-      <c r="D335" t="inlineStr">
-        <is>
-          <t>V0710349973</t>
-        </is>
-      </c>
+      <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
           <t>9903.03.01</t>
@@ -28432,17 +28432,17 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>2566100</t>
+          <t>2615771</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>EF4-0232282-2</t>
+          <t>EF4-0232406-7</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
+          <t>Vessel, Non-container</t>
         </is>
       </c>
       <c r="D336" t="inlineStr"/>
@@ -28468,27 +28468,27 @@
       </c>
       <c r="I336" t="inlineStr">
         <is>
-          <t>4811.59.4040</t>
+          <t>8210.00.0000</t>
         </is>
       </c>
       <c r="J336" t="inlineStr">
         <is>
-          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+          <t>COVE HOME LLC</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
         <is>
-          <t>BAULIN</t>
+          <t>COVHOM01</t>
         </is>
       </c>
       <c r="L336" t="inlineStr">
         <is>
-          <t>56-193913400</t>
+          <t>30-136116600</t>
         </is>
       </c>
       <c r="M336" t="inlineStr">
         <is>
-          <t>2026-06-21 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
       <c r="N336" t="inlineStr">
@@ -28498,34 +28498,34 @@
       </c>
       <c r="O336" t="inlineStr">
         <is>
-          <t>SURTECO GMBH</t>
+          <t>P. IONNOU G ZARKADIS QE</t>
         </is>
       </c>
       <c r="P336" t="inlineStr">
         <is>
-          <t>SURTECO GMBH</t>
+          <t>P. IONNOU G ZARKADIS QE</t>
         </is>
       </c>
       <c r="Q336" t="inlineStr">
         <is>
-          <t>2026-06-01 00:00:00</t>
+          <t>2026-06-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>2566100</t>
+          <t>2615771</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>EF4-0232282-2</t>
+          <t>EF4-0232406-7</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
+          <t>Vessel, Non-container</t>
         </is>
       </c>
       <c r="D337" t="inlineStr"/>
@@ -28551,27 +28551,27 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>4811.59.4040</t>
+          <t>8210.00.0000</t>
         </is>
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+          <t>COVE HOME LLC</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
         <is>
-          <t>BAULIN</t>
+          <t>COVHOM01</t>
         </is>
       </c>
       <c r="L337" t="inlineStr">
         <is>
-          <t>56-193913400</t>
+          <t>30-136116600</t>
         </is>
       </c>
       <c r="M337" t="inlineStr">
         <is>
-          <t>2026-06-21 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
       <c r="N337" t="inlineStr">
@@ -28581,29 +28581,29 @@
       </c>
       <c r="O337" t="inlineStr">
         <is>
-          <t>SURTECO GMBH</t>
+          <t>P. IONNOU G ZARKADIS QE</t>
         </is>
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t>SURTECO GMBH</t>
+          <t>P. IONNOU G ZARKADIS QE</t>
         </is>
       </c>
       <c r="Q337" t="inlineStr">
         <is>
-          <t>2026-06-01 00:00:00</t>
+          <t>2026-06-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>2566100</t>
+          <t>2565847</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>EF4-0232282-2</t>
+          <t>EF4-0231725-1</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -28624,7 +28624,7 @@
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H338" t="inlineStr">
@@ -28634,64 +28634,64 @@
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>4811.59.4040</t>
+          <t>5407.20.0000</t>
         </is>
       </c>
       <c r="J338" t="inlineStr">
         <is>
-          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+          <t>VEER CORPORATIONS INC</t>
         </is>
       </c>
       <c r="K338" t="inlineStr">
         <is>
-          <t>BAULIN</t>
+          <t>VEECOR01</t>
         </is>
       </c>
       <c r="L338" t="inlineStr">
         <is>
-          <t>56-193913400</t>
+          <t>99-106989200</t>
         </is>
       </c>
       <c r="M338" t="inlineStr">
         <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="N338" t="inlineStr">
+        <is>
           <t>2026-06-21 00:00:00</t>
         </is>
       </c>
-      <c r="N338" t="inlineStr">
-        <is>
-          <t>2026-06-20 00:00:00</t>
-        </is>
-      </c>
       <c r="O338" t="inlineStr">
         <is>
-          <t>SURTECO GMBH</t>
+          <t>VEER PLASTIC PVT LTD</t>
         </is>
       </c>
       <c r="P338" t="inlineStr">
         <is>
-          <t>SURTECO GMBH</t>
+          <t>VEER PLASTIC PVT LTD</t>
         </is>
       </c>
       <c r="Q338" t="inlineStr">
         <is>
-          <t>2026-06-01 00:00:00</t>
+          <t>2026-05-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>2615771</t>
+          <t>2565848</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>EF4-0232406-7</t>
+          <t>EF4-0231726-9</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Vessel, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D339" t="inlineStr"/>
@@ -28717,64 +28717,64 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>8210.00.0000</t>
+          <t>5603.14.9090</t>
         </is>
       </c>
       <c r="J339" t="inlineStr">
         <is>
-          <t>COVE HOME LLC</t>
+          <t>VEER CORPORATIONS INC</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>COVHOM01</t>
+          <t>VEECOR01</t>
         </is>
       </c>
       <c r="L339" t="inlineStr">
         <is>
-          <t>30-136116600</t>
+          <t>99-106989200</t>
         </is>
       </c>
       <c r="M339" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-19 00:00:00</t>
         </is>
       </c>
       <c r="N339" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-21 00:00:00</t>
         </is>
       </c>
       <c r="O339" t="inlineStr">
         <is>
-          <t>P. IONNOU G ZARKADIS QE</t>
+          <t>VEER PLASTIC PVT LTD</t>
         </is>
       </c>
       <c r="P339" t="inlineStr">
         <is>
-          <t>P. IONNOU G ZARKADIS QE</t>
+          <t>VEER PLASTIC PVT LTD</t>
         </is>
       </c>
       <c r="Q339" t="inlineStr">
         <is>
-          <t>2026-06-06 00:00:00</t>
+          <t>2026-05-11 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>2615771</t>
+          <t>2565849</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>EF4-0232406-7</t>
+          <t>EF4-0231727-7</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Vessel, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D340" t="inlineStr"/>
@@ -28790,55 +28790,1142 @@
       </c>
       <c r="G340" t="inlineStr">
         <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="N340" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O340" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P340" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q340" t="inlineStr">
+        <is>
+          <t>2026-05-11 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2565891</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>EF4-0231922-4</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr"/>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N341" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O341" t="inlineStr">
+        <is>
+          <t>SEDAMYL UK</t>
+        </is>
+      </c>
+      <c r="P341" t="inlineStr">
+        <is>
+          <t>SEDAMYL UK</t>
+        </is>
+      </c>
+      <c r="Q341" t="inlineStr">
+        <is>
+          <t>2026-05-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2565934</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>EF4-0231991-9</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>V0710339289</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N342" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O342" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P342" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q342" t="inlineStr">
+        <is>
+          <t>2026-05-18 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2566075</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>EF4-0232185-7</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>V0710339289</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>9903.82.01,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="N343" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O343" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P343" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q343" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2566102</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>EF4-0232187-3</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr"/>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>9903.82.22,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="N344" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O344" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P344" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q344" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2565923</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>EF4-0232195-6</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr"/>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>9903.91.01</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>ARTS, PRDS OF CN SUB(B)US NT31</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>9903.91.01</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.02,7228.30.6000</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>MAHA USA LLC</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>MAHUSA</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>52-213556300</t>
+        </is>
+      </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N345" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O345" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="P345" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="Q345" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2565923</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>EF4-0232195-6</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr"/>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
           <t>002</t>
         </is>
       </c>
-      <c r="H340" t="inlineStr">
-        <is>
-          <t>9903.03.01</t>
-        </is>
-      </c>
-      <c r="I340" t="inlineStr">
-        <is>
-          <t>8210.00.0000</t>
-        </is>
-      </c>
-      <c r="J340" t="inlineStr">
-        <is>
-          <t>COVE HOME LLC</t>
-        </is>
-      </c>
-      <c r="K340" t="inlineStr">
-        <is>
-          <t>COVHOM01</t>
-        </is>
-      </c>
-      <c r="L340" t="inlineStr">
-        <is>
-          <t>30-136116600</t>
-        </is>
-      </c>
-      <c r="M340" t="inlineStr">
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>9903.82.02,7215.50.0016</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>MAHA USA LLC</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>MAHUSA</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>52-213556300</t>
+        </is>
+      </c>
+      <c r="M346" t="inlineStr">
         <is>
           <t>2026-06-20 00:00:00</t>
         </is>
       </c>
-      <c r="N340" t="inlineStr">
+      <c r="N346" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O346" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="P346" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="Q346" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2565923</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>EF4-0232195-6</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr"/>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>9903.82.02,7216.33.0090</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>MAHA USA LLC</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>MAHUSA</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>52-213556300</t>
+        </is>
+      </c>
+      <c r="M347" t="inlineStr">
         <is>
           <t>2026-06-20 00:00:00</t>
         </is>
       </c>
-      <c r="O340" t="inlineStr">
-        <is>
-          <t>P. IONNOU G ZARKADIS QE</t>
-        </is>
-      </c>
-      <c r="P340" t="inlineStr">
-        <is>
-          <t>P. IONNOU G ZARKADIS QE</t>
-        </is>
-      </c>
-      <c r="Q340" t="inlineStr">
+      <c r="N347" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O347" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="P347" t="inlineStr">
+        <is>
+          <t>THYSSENKRUPP SCHULTE GMBH</t>
+        </is>
+      </c>
+      <c r="Q347" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2566146</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>EF4-0232246-7</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr"/>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>1109.00.9010</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="N348" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O348" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="P348" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="Q348" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2566173</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>EF4-0232274-9</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr"/>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N349" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O349" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P349" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q349" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2565864</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>EF4-0232315-0</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr"/>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N350" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O350" t="inlineStr">
+        <is>
+          <t>ROQUETTE FRERES</t>
+        </is>
+      </c>
+      <c r="P350" t="inlineStr">
+        <is>
+          <t>ROQUETTE FRERES</t>
+        </is>
+      </c>
+      <c r="Q350" t="inlineStr">
+        <is>
+          <t>2026-05-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2566183</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>EF4-0232343-2</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr"/>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>2106.90.9998</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="N351" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O351" t="inlineStr">
+        <is>
+          <t>IRCA SRL</t>
+        </is>
+      </c>
+      <c r="P351" t="inlineStr">
+        <is>
+          <t>IRCA SRL</t>
+        </is>
+      </c>
+      <c r="Q351" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2566264</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>EF4-0232584-1</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr"/>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>3815.90.5000</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>JOBACHEM CORPORATION</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>JOBLP01</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>32-052169200</t>
+        </is>
+      </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="N352" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O352" t="inlineStr">
+        <is>
+          <t>JOBACHEM GMBH</t>
+        </is>
+      </c>
+      <c r="P352" t="inlineStr">
+        <is>
+          <t>JOBACHEM GMBH</t>
+        </is>
+      </c>
+      <c r="Q352" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2566264</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>EF4-0232584-1</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr"/>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>2916.14.2050</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>JOBACHEM CORPORATION</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>JOBLP01</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>32-052169200</t>
+        </is>
+      </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>2026-06-22 00:00:00</t>
+        </is>
+      </c>
+      <c r="N353" t="inlineStr">
+        <is>
+          <t>2026-06-21 00:00:00</t>
+        </is>
+      </c>
+      <c r="O353" t="inlineStr">
+        <is>
+          <t>JOBACHEM GMBH</t>
+        </is>
+      </c>
+      <c r="P353" t="inlineStr">
+        <is>
+          <t>JOBACHEM GMBH</t>
+        </is>
+      </c>
+      <c r="Q353" t="inlineStr">
         <is>
           <t>2026-06-06 00:00:00</t>
         </is>

</xml_diff>

<commit_message>
Append trimika data — 11 new rows, 389 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q379"/>
+  <dimension ref="A1:Q390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32149,6 +32149,931 @@
         </is>
       </c>
     </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2565850</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>EF4-0231705-3</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr"/>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q380" t="inlineStr">
+        <is>
+          <t>2026-05-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2565826</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>EF4-0231707-9</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr"/>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P381" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q381" t="inlineStr">
+        <is>
+          <t>2026-04-21 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2565828</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>EF4-0231712-9</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr"/>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N382" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P382" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q382" t="inlineStr">
+        <is>
+          <t>2026-05-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2565829</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>EF4-0231713-7</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr"/>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P383" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q383" t="inlineStr">
+        <is>
+          <t>2026-05-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2565908</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>EF4-0232026-3</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr"/>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1061</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P384" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q384" t="inlineStr">
+        <is>
+          <t>2026-05-09 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2566016</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>EF4-0232063-6</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr"/>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N385" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P385" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q385" t="inlineStr">
+        <is>
+          <t>2026-05-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2566041</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>EF4-0232085-9</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr"/>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8302.42.3015</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>GRASS AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>GRAAME</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>51-066023000</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N386" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t>SACA PRECISION LTD</t>
+        </is>
+      </c>
+      <c r="P386" t="inlineStr">
+        <is>
+          <t>SACA PRECISION LTD</t>
+        </is>
+      </c>
+      <c r="Q386" t="inlineStr">
+        <is>
+          <t>2026-05-21 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2565946</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>EF4-0232241-8</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>V1626464484</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr"/>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N387" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIAC</t>
+        </is>
+      </c>
+      <c r="P387" t="inlineStr">
+        <is>
+          <t>PRZEDSIEBIORSTWO PRZEMYSLU ZIEMNIACZANEGO PEPEES S.A.</t>
+        </is>
+      </c>
+      <c r="Q387" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>4539555</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>EF4-0232777-1</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>V1626464484</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>3926.90.6090</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>ESBAND USA INC</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>ESBUSA01</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>87-443503100</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t>MAX SCHLATTERER</t>
+        </is>
+      </c>
+      <c r="P388" t="inlineStr">
+        <is>
+          <t>MAX SCHLATTERER</t>
+        </is>
+      </c>
+      <c r="Q388" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>4539555</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>EF4-0232777-1</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>V1626464484</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>4010.35.9000</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>ESBAND USA INC</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>ESBUSA01</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>87-443503100</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t>MAX SCHLATTERER</t>
+        </is>
+      </c>
+      <c r="P389" t="inlineStr">
+        <is>
+          <t>MAX SCHLATTERER</t>
+        </is>
+      </c>
+      <c r="Q389" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>4539555</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>EF4-0232777-1</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>V1626464484</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>5910.00.1090</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>ESBAND USA INC</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>ESBUSA01</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>87-443503100</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t>MAX SCHLATTERER</t>
+        </is>
+      </c>
+      <c r="P390" t="inlineStr">
+        <is>
+          <t>MAX SCHLATTERER</t>
+        </is>
+      </c>
+      <c r="Q390" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 22 new rows, 411 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q390"/>
+  <dimension ref="A1:Q412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33074,6 +33074,1808 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2565903</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>EF4-0231899-4</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr"/>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P391" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q391" t="inlineStr">
+        <is>
+          <t>2026-05-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2566026</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>EF4-0232031-3</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>V2108743882</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>8436.80.0020</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>MDE MACHINERY INC</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>MDEMAC02</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>38-438331300</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+      <c r="N392" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t>MDE MACHINERY LTD</t>
+        </is>
+      </c>
+      <c r="P392" t="inlineStr">
+        <is>
+          <t>MDE MACHINERY LTD</t>
+        </is>
+      </c>
+      <c r="Q392" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2565097</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>EF4-0232240-0</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>V2108743882</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr"/>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>1108.12.0010</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="P393" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="Q393" t="inlineStr">
+        <is>
+          <t>2026-03-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2566241</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>EF4-0232379-6</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr"/>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>6913.90.1000</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>MESO CASA LLC</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>MESCAS01</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>93-375253000</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>ATUTO S DE R.L.</t>
+        </is>
+      </c>
+      <c r="P394" t="inlineStr">
+        <is>
+          <t>ATUTO S DE R.L.</t>
+        </is>
+      </c>
+      <c r="Q394" t="inlineStr">
+        <is>
+          <t>2026-06-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2566241</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>EF4-0232379-6</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr"/>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>4420.11.0090</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>MESO CASA LLC</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>MESCAS01</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>93-375253000</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>2026-06-18 00:00:00</t>
+        </is>
+      </c>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>ATUTO S DE R.L.</t>
+        </is>
+      </c>
+      <c r="P395" t="inlineStr">
+        <is>
+          <t>ATUTO S DE R.L.</t>
+        </is>
+      </c>
+      <c r="Q395" t="inlineStr">
+        <is>
+          <t>2026-06-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2566258</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>EF4-0232463-8</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr"/>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>3920.61.0000</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>TUBUS BAUER GMBH</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>TUBBAU01</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>091601-00584</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>TUBUS BAUER GMBH</t>
+        </is>
+      </c>
+      <c r="P396" t="inlineStr">
+        <is>
+          <t>TUBUS BAUER GMBH</t>
+        </is>
+      </c>
+      <c r="Q396" t="inlineStr">
+        <is>
+          <t>2026-06-09 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>105504778</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>EF4-0232476-0</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr"/>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr"/>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P397" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q397" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>105504780</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>EF4-0232486-9</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr"/>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr"/>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P398" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q398" t="inlineStr">
+        <is>
+          <t>2026-06-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2566249</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>EF4-0232524-7</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr"/>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P399" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q399" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2566249</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>EF4-0232524-7</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr"/>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P400" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q400" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2566249</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>EF4-0232524-7</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr"/>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P401" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q401" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2566249</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>EF4-0232524-7</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr"/>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5160</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P402" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q402" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>105504788</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>EF4-0232545-2</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr"/>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr"/>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>VOLVO CARS GHENT</t>
+        </is>
+      </c>
+      <c r="P403" t="inlineStr">
+        <is>
+          <t>VOLVO CARS GHENT</t>
+        </is>
+      </c>
+      <c r="Q403" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>105504789</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>EF4-0232555-1</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr"/>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr"/>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>VOLVO CARS GHENT</t>
+        </is>
+      </c>
+      <c r="P404" t="inlineStr">
+        <is>
+          <t>VOLVO CARS GHENT</t>
+        </is>
+      </c>
+      <c r="Q404" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>105504791</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>EF4-0232565-0</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr"/>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr"/>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P405" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q405" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>105504792</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>EF4-0232567-6</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr"/>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr"/>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P406" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q406" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>105504793</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>EF4-0232569-2</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr"/>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr"/>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P407" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q407" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>105504795</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>EF4-0232583-3</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr"/>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr"/>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="P408" t="inlineStr">
+        <is>
+          <t>VOLVO CAR INTERNATIONAL CORPORATION</t>
+        </is>
+      </c>
+      <c r="Q408" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>105504796</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>EF4-0232585-8</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr"/>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr"/>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>IFF, INC.</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>58-149385700</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>VOLVO CARS GHENT</t>
+        </is>
+      </c>
+      <c r="P409" t="inlineStr">
+        <is>
+          <t>VOLVO CARS GHENT</t>
+        </is>
+      </c>
+      <c r="Q409" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2566322</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>EF4-0232612-0</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr"/>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>8419.19.0120</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>THERMAL PROCESS DEVELOPMENT LLC</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>THEPRO01</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>82-175198100</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>INTEC ENGINEERING GMBH</t>
+        </is>
+      </c>
+      <c r="P410" t="inlineStr">
+        <is>
+          <t>INTEC ENGINEERING GMBH</t>
+        </is>
+      </c>
+      <c r="Q410" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>4539557</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>EF4-0232785-4</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>709758804</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>8438.90.9060</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>CANTRELL GAINCO GROUP INC</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>CANGAI01</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>31-151121700</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="P411" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="Q411" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>4539561</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>EF4-0232788-8</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>709758804</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>4010.19.9100</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>CANTRELL GAINCO GROUP INC</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>CANGAI01</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>31-151121700</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>MANIFATTURE TECNICHE INDUSTRIALI SA</t>
+        </is>
+      </c>
+      <c r="P412" t="inlineStr">
+        <is>
+          <t>MANIFATTURE TECNICHE INDUSTRIALI SA</t>
+        </is>
+      </c>
+      <c r="Q412" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 3 new rows, 414 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q412"/>
+  <dimension ref="A1:Q415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34876,6 +34876,255 @@
         </is>
       </c>
     </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2566151</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>EF4-0232363-0</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr"/>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t>SEDAMYL UK</t>
+        </is>
+      </c>
+      <c r="P413" t="inlineStr">
+        <is>
+          <t>SEDAMYL UK</t>
+        </is>
+      </c>
+      <c r="Q413" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2566238</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>EF4-0232707-8</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr"/>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="N414" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t>CARGILL BARBY</t>
+        </is>
+      </c>
+      <c r="P414" t="inlineStr">
+        <is>
+          <t>CARGILL BARBY</t>
+        </is>
+      </c>
+      <c r="Q414" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2566351</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>EF4-0232708-6</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr"/>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="N415" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t>CARGILL BARBY</t>
+        </is>
+      </c>
+      <c r="P415" t="inlineStr">
+        <is>
+          <t>CARGILL BARBY</t>
+        </is>
+      </c>
+      <c r="Q415" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 10 new rows, 432 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q423"/>
+  <dimension ref="A1:Q433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35813,6 +35813,856 @@
         </is>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2565881</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>EF4-0231827-5</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr"/>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8302.42.3065</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>GRASS AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>GRAAME</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>51-066023000</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="N424" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t>BAIHUI ENTERPRISE(KAISI)</t>
+        </is>
+      </c>
+      <c r="P424" t="inlineStr">
+        <is>
+          <t>BAIHUI ENTERPRISE(KAISI)</t>
+        </is>
+      </c>
+      <c r="Q424" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2565881</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>EF4-0231827-5</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr"/>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.30.5000</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>GRASS AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>GRAAME</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>51-066023000</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+      <c r="N425" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t>BAIHUI ENTERPRISE(KAISI)</t>
+        </is>
+      </c>
+      <c r="P425" t="inlineStr">
+        <is>
+          <t>BAIHUI ENTERPRISE(KAISI)</t>
+        </is>
+      </c>
+      <c r="Q425" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2566043</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>EF4-0232123-8</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr"/>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="N426" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P426" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q426" t="inlineStr">
+        <is>
+          <t>2026-05-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2566085</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>EF4-0232125-3</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>V0710342853</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="N427" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P427" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q427" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2566136</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>EF4-0232217-8</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>V0710342853</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>ROQUETTE FRERES</t>
+        </is>
+      </c>
+      <c r="P428" t="inlineStr">
+        <is>
+          <t>ROQUETTE FRERES</t>
+        </is>
+      </c>
+      <c r="Q428" t="inlineStr">
+        <is>
+          <t>2026-05-30 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>2566037</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>EF4-0232303-6</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>V1P06267054</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>1108.14.0000</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>2026-06-30 00:00:00</t>
+        </is>
+      </c>
+      <c r="N429" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="P429" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="Q429" t="inlineStr">
+        <is>
+          <t>2026-05-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2566247</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>EF4-0232455-4</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>V1P06267054</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P430" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q430" t="inlineStr">
+        <is>
+          <t>2026-06-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2566232</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>EF4-0232576-7</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr"/>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>3920.20.0055</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>TEUFELBERGER G.E.S.M.B.H</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>TEUSEI01</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>181704-13780</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t>TEUFELBERGER GMBH</t>
+        </is>
+      </c>
+      <c r="P431" t="inlineStr">
+        <is>
+          <t>TEUFELBERGER GMBH</t>
+        </is>
+      </c>
+      <c r="Q431" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>4539529</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>EF4-0232822-5</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr"/>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>9903.03.01,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t>XIAMEN CUBES INDUSTRIAL &amp; TRADING C</t>
+        </is>
+      </c>
+      <c r="P432" t="inlineStr">
+        <is>
+          <t>XIAMEN CUBES INDUSTRIAL &amp; TRADING C</t>
+        </is>
+      </c>
+      <c r="Q432" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>4539572</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>EF4-0232838-1</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>711583181</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>8438.90.9060</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>CANTRELL GAINCO GROUP INC</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>CANGAI01</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>31-151121700</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>2026-06-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="P433" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="Q433" t="inlineStr">
+        <is>
+          <t>2026-06-26 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 15 new rows, 800 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q786"/>
+  <dimension ref="A1:Q801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66162,6 +66162,1251 @@
         </is>
       </c>
     </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2566022</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>EF4-0232169-1</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr"/>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>3920.62.0090</t>
+        </is>
+      </c>
+      <c r="J787" t="inlineStr">
+        <is>
+          <t>GULF ATLANTIC PACKAGING CORP</t>
+        </is>
+      </c>
+      <c r="K787" t="inlineStr">
+        <is>
+          <t>GULATL</t>
+        </is>
+      </c>
+      <c r="L787" t="inlineStr">
+        <is>
+          <t>58-184378700</t>
+        </is>
+      </c>
+      <c r="M787" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N787" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O787" t="inlineStr">
+        <is>
+          <t>CONSENT FZCO</t>
+        </is>
+      </c>
+      <c r="P787" t="inlineStr">
+        <is>
+          <t>CONSENT FZCO</t>
+        </is>
+      </c>
+      <c r="Q787" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2566099</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>EF4-0232186-5</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr"/>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>9903.82.22,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J788" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K788" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L788" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M788" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N788" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O788" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P788" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q788" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2566099</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>EF4-0232186-5</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr"/>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>9903.82.22,8431.20.0000</t>
+        </is>
+      </c>
+      <c r="J789" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K789" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L789" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M789" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N789" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O789" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P789" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q789" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2565995</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>EF4-0232279-8</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr"/>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>9903.03.01,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J790" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K790" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L790" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M790" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N790" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O790" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P790" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q790" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2565995</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>EF4-0232279-8</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr"/>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J791" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K791" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L791" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M791" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N791" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O791" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P791" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q791" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2565996</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>EF4-0232280-6</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr"/>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J792" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L792" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M792" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N792" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O792" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P792" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q792" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2565996</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>EF4-0232280-6</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr"/>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>9903.03.01,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K793" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L793" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M793" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N793" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O793" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P793" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q793" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2565996</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>EF4-0232280-6</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr"/>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8302.42.3065</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K794" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L794" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M794" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N794" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O794" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P794" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q794" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2565996</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>EF4-0232280-6</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr"/>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,9403.20.0075</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K795" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L795" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M795" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N795" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O795" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P795" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q795" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2565996</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>EF4-0232280-6</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr"/>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>9903.03.01,9903.76.04,9403.91.0080</t>
+        </is>
+      </c>
+      <c r="J796" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K796" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L796" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M796" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N796" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O796" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P796" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q796" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2566367</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>EF4-0232744-1</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr"/>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J797" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K797" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L797" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M797" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N797" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O797" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P797" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q797" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2566367</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>EF4-0232744-1</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr"/>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J798" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K798" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L798" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M798" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N798" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O798" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P798" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q798" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2566367</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>EF4-0232744-1</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr"/>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J799" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K799" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L799" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M799" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N799" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O799" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P799" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q799" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2566367</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>EF4-0232744-1</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr"/>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J800" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K800" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L800" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M800" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N800" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O800" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P800" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q800" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2566367</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>EF4-0232744-1</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr"/>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J801" t="inlineStr">
+        <is>
+          <t>BORGERS USA CORP</t>
+        </is>
+      </c>
+      <c r="K801" t="inlineStr">
+        <is>
+          <t>BORUSA</t>
+        </is>
+      </c>
+      <c r="L801" t="inlineStr">
+        <is>
+          <t>65-117296500</t>
+        </is>
+      </c>
+      <c r="M801" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="N801" t="inlineStr">
+        <is>
+          <t>2026-07-02 00:00:00</t>
+        </is>
+      </c>
+      <c r="O801" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="P801" t="inlineStr">
+        <is>
+          <t>AUTONEUM CZ S.R.O.</t>
+        </is>
+      </c>
+      <c r="Q801" t="inlineStr">
+        <is>
+          <t>2026-06-20 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 10 new rows, 803 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q801"/>
+  <dimension ref="A1:Q804"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66414,12 +66414,12 @@
     <row r="790">
       <c r="A790" t="inlineStr">
         <is>
-          <t>2565995</t>
+          <t>2566367</t>
         </is>
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>EF4-0232279-8</t>
+          <t>EF4-0232744-1</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -66430,12 +66430,12 @@
       <c r="D790" t="inlineStr"/>
       <c r="E790" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F790" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G790" t="inlineStr">
@@ -66445,32 +66445,32 @@
       </c>
       <c r="H790" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I790" t="inlineStr">
         <is>
-          <t>9903.03.01,9403.99.9045</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J790" t="inlineStr">
         <is>
-          <t>VISUAL CREATIONS, INC.</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K790" t="inlineStr">
         <is>
-          <t>VISCRE</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L790" t="inlineStr">
         <is>
-          <t>20-461602300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M790" t="inlineStr">
         <is>
-          <t>2026-07-04 00:00:00</t>
+          <t>2026-07-02 00:00:00</t>
         </is>
       </c>
       <c r="N790" t="inlineStr">
@@ -66480,29 +66480,29 @@
       </c>
       <c r="O790" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P790" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q790" t="inlineStr">
         <is>
-          <t>2026-06-02 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" t="inlineStr">
         <is>
-          <t>2565995</t>
+          <t>2566367</t>
         </is>
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>EF4-0232279-8</t>
+          <t>EF4-0232744-1</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
@@ -66513,12 +66513,12 @@
       <c r="D791" t="inlineStr"/>
       <c r="E791" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G791" t="inlineStr">
@@ -66528,32 +66528,32 @@
       </c>
       <c r="H791" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I791" t="inlineStr">
         <is>
-          <t>9903.03.01,3926.90.9989</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J791" t="inlineStr">
         <is>
-          <t>VISUAL CREATIONS, INC.</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K791" t="inlineStr">
         <is>
-          <t>VISCRE</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L791" t="inlineStr">
         <is>
-          <t>20-461602300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M791" t="inlineStr">
         <is>
-          <t>2026-07-04 00:00:00</t>
+          <t>2026-07-02 00:00:00</t>
         </is>
       </c>
       <c r="N791" t="inlineStr">
@@ -66563,29 +66563,29 @@
       </c>
       <c r="O791" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P791" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q791" t="inlineStr">
         <is>
-          <t>2026-06-02 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="792">
       <c r="A792" t="inlineStr">
         <is>
-          <t>2565996</t>
+          <t>2566367</t>
         </is>
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>EF4-0232280-6</t>
+          <t>EF4-0232744-1</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -66596,47 +66596,47 @@
       <c r="D792" t="inlineStr"/>
       <c r="E792" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F792" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G792" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
         <is>
-          <t>9903.03.01,3926.90.9989</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J792" t="inlineStr">
         <is>
-          <t>VISUAL CREATIONS, INC.</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K792" t="inlineStr">
         <is>
-          <t>VISCRE</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L792" t="inlineStr">
         <is>
-          <t>20-461602300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M792" t="inlineStr">
         <is>
-          <t>2026-07-04 00:00:00</t>
+          <t>2026-07-02 00:00:00</t>
         </is>
       </c>
       <c r="N792" t="inlineStr">
@@ -66646,29 +66646,29 @@
       </c>
       <c r="O792" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P792" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q792" t="inlineStr">
         <is>
-          <t>2026-06-02 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
         <is>
-          <t>2565996</t>
+          <t>2566367</t>
         </is>
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>EF4-0232280-6</t>
+          <t>EF4-0232744-1</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
@@ -66679,47 +66679,47 @@
       <c r="D793" t="inlineStr"/>
       <c r="E793" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G793" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
         <is>
-          <t>9903.03.01,9403.99.9045</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J793" t="inlineStr">
         <is>
-          <t>VISUAL CREATIONS, INC.</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K793" t="inlineStr">
         <is>
-          <t>VISCRE</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L793" t="inlineStr">
         <is>
-          <t>20-461602300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M793" t="inlineStr">
         <is>
-          <t>2026-07-04 00:00:00</t>
+          <t>2026-07-02 00:00:00</t>
         </is>
       </c>
       <c r="N793" t="inlineStr">
@@ -66729,29 +66729,29 @@
       </c>
       <c r="O793" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P793" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q793" t="inlineStr">
         <is>
-          <t>2026-06-02 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="794">
       <c r="A794" t="inlineStr">
         <is>
-          <t>2565996</t>
+          <t>2566367</t>
         </is>
       </c>
       <c r="B794" t="inlineStr">
         <is>
-          <t>EF4-0232280-6</t>
+          <t>EF4-0232744-1</t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
@@ -66762,47 +66762,47 @@
       <c r="D794" t="inlineStr"/>
       <c r="E794" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F794" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G794" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>005</t>
         </is>
       </c>
       <c r="H794" t="inlineStr">
         <is>
-          <t>9903.88.15</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I794" t="inlineStr">
         <is>
-          <t>9903.03.06,9903.82.09,8302.42.3065</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J794" t="inlineStr">
         <is>
-          <t>VISUAL CREATIONS, INC.</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K794" t="inlineStr">
         <is>
-          <t>VISCRE</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L794" t="inlineStr">
         <is>
-          <t>20-461602300</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M794" t="inlineStr">
         <is>
-          <t>2026-07-04 00:00:00</t>
+          <t>2026-07-02 00:00:00</t>
         </is>
       </c>
       <c r="N794" t="inlineStr">
@@ -66812,29 +66812,29 @@
       </c>
       <c r="O794" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P794" t="inlineStr">
         <is>
-          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q794" t="inlineStr">
         <is>
-          <t>2026-06-02 00:00:00</t>
+          <t>2026-06-20 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
         <is>
-          <t>2565996</t>
+          <t>2565995</t>
         </is>
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>EF4-0232280-6</t>
+          <t>EF4-0232279-8</t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
@@ -66855,7 +66855,7 @@
       </c>
       <c r="G795" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H795" t="inlineStr">
@@ -66865,7 +66865,7 @@
       </c>
       <c r="I795" t="inlineStr">
         <is>
-          <t>9903.03.06,9903.82.09,9403.20.0075</t>
+          <t>9903.03.01,9403.99.9045</t>
         </is>
       </c>
       <c r="J795" t="inlineStr">
@@ -66890,7 +66890,7 @@
       </c>
       <c r="N795" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O795" t="inlineStr">
@@ -66912,12 +66912,12 @@
     <row r="796">
       <c r="A796" t="inlineStr">
         <is>
-          <t>2565996</t>
+          <t>2565995</t>
         </is>
       </c>
       <c r="B796" t="inlineStr">
         <is>
-          <t>EF4-0232280-6</t>
+          <t>EF4-0232279-8</t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
@@ -66928,27 +66928,27 @@
       <c r="D796" t="inlineStr"/>
       <c r="E796" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="F796" t="inlineStr">
         <is>
-          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
         </is>
       </c>
       <c r="G796" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H796" t="inlineStr">
         <is>
-          <t>9903.88.03</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="I796" t="inlineStr">
         <is>
-          <t>9903.03.01,9903.76.04,9403.91.0080</t>
+          <t>9903.03.01,3926.90.9989</t>
         </is>
       </c>
       <c r="J796" t="inlineStr">
@@ -66973,7 +66973,7 @@
       </c>
       <c r="N796" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O796" t="inlineStr">
@@ -66995,12 +66995,12 @@
     <row r="797">
       <c r="A797" t="inlineStr">
         <is>
-          <t>2566367</t>
+          <t>2565996</t>
         </is>
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>EF4-0232744-1</t>
+          <t>EF4-0232280-6</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
@@ -67011,12 +67011,12 @@
       <c r="D797" t="inlineStr"/>
       <c r="E797" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="F797" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
         </is>
       </c>
       <c r="G797" t="inlineStr">
@@ -67026,64 +67026,64 @@
       </c>
       <c r="H797" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="I797" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+          <t>9903.03.01,3926.90.9989</t>
         </is>
       </c>
       <c r="J797" t="inlineStr">
         <is>
-          <t>BORGERS USA CORP</t>
+          <t>VISUAL CREATIONS, INC.</t>
         </is>
       </c>
       <c r="K797" t="inlineStr">
         <is>
-          <t>BORUSA</t>
+          <t>VISCRE</t>
         </is>
       </c>
       <c r="L797" t="inlineStr">
         <is>
-          <t>65-117296500</t>
+          <t>20-461602300</t>
         </is>
       </c>
       <c r="M797" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="N797" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O797" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="P797" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="Q797" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-02 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr">
         <is>
-          <t>2566367</t>
+          <t>2565996</t>
         </is>
       </c>
       <c r="B798" t="inlineStr">
         <is>
-          <t>EF4-0232744-1</t>
+          <t>EF4-0232280-6</t>
         </is>
       </c>
       <c r="C798" t="inlineStr">
@@ -67094,12 +67094,12 @@
       <c r="D798" t="inlineStr"/>
       <c r="E798" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="F798" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
         </is>
       </c>
       <c r="G798" t="inlineStr">
@@ -67109,64 +67109,64 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+          <t>9903.03.01,9403.99.9045</t>
         </is>
       </c>
       <c r="J798" t="inlineStr">
         <is>
-          <t>BORGERS USA CORP</t>
+          <t>VISUAL CREATIONS, INC.</t>
         </is>
       </c>
       <c r="K798" t="inlineStr">
         <is>
-          <t>BORUSA</t>
+          <t>VISCRE</t>
         </is>
       </c>
       <c r="L798" t="inlineStr">
         <is>
-          <t>65-117296500</t>
+          <t>20-461602300</t>
         </is>
       </c>
       <c r="M798" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="N798" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O798" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="P798" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="Q798" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-02 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
         <is>
-          <t>2566367</t>
+          <t>2565996</t>
         </is>
       </c>
       <c r="B799" t="inlineStr">
         <is>
-          <t>EF4-0232744-1</t>
+          <t>EF4-0232280-6</t>
         </is>
       </c>
       <c r="C799" t="inlineStr">
@@ -67177,12 +67177,12 @@
       <c r="D799" t="inlineStr"/>
       <c r="E799" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="F799" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
         </is>
       </c>
       <c r="G799" t="inlineStr">
@@ -67192,64 +67192,64 @@
       </c>
       <c r="H799" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.15</t>
         </is>
       </c>
       <c r="I799" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+          <t>9903.03.06,9903.82.09,8302.42.3065</t>
         </is>
       </c>
       <c r="J799" t="inlineStr">
         <is>
-          <t>BORGERS USA CORP</t>
+          <t>VISUAL CREATIONS, INC.</t>
         </is>
       </c>
       <c r="K799" t="inlineStr">
         <is>
-          <t>BORUSA</t>
+          <t>VISCRE</t>
         </is>
       </c>
       <c r="L799" t="inlineStr">
         <is>
-          <t>65-117296500</t>
+          <t>20-461602300</t>
         </is>
       </c>
       <c r="M799" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="N799" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O799" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="P799" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="Q799" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-02 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="800">
       <c r="A800" t="inlineStr">
         <is>
-          <t>2566367</t>
+          <t>2565996</t>
         </is>
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t>EF4-0232744-1</t>
+          <t>EF4-0232280-6</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
@@ -67260,12 +67260,12 @@
       <c r="D800" t="inlineStr"/>
       <c r="E800" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="F800" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
         </is>
       </c>
       <c r="G800" t="inlineStr">
@@ -67275,64 +67275,64 @@
       </c>
       <c r="H800" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="I800" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+          <t>9903.03.06,9903.82.09,9403.20.0075</t>
         </is>
       </c>
       <c r="J800" t="inlineStr">
         <is>
-          <t>BORGERS USA CORP</t>
+          <t>VISUAL CREATIONS, INC.</t>
         </is>
       </c>
       <c r="K800" t="inlineStr">
         <is>
-          <t>BORUSA</t>
+          <t>VISCRE</t>
         </is>
       </c>
       <c r="L800" t="inlineStr">
         <is>
-          <t>65-117296500</t>
+          <t>20-461602300</t>
         </is>
       </c>
       <c r="M800" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="N800" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O800" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="P800" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="Q800" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-02 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="801">
       <c r="A801" t="inlineStr">
         <is>
-          <t>2566367</t>
+          <t>2565996</t>
         </is>
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t>EF4-0232744-1</t>
+          <t>EF4-0232280-6</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
@@ -67343,12 +67343,12 @@
       <c r="D801" t="inlineStr"/>
       <c r="E801" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="F801" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
         </is>
       </c>
       <c r="G801" t="inlineStr">
@@ -67358,52 +67358,301 @@
       </c>
       <c r="H801" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.88.03</t>
         </is>
       </c>
       <c r="I801" t="inlineStr">
         <is>
-          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+          <t>9903.03.01,9903.76.04,9403.91.0080</t>
         </is>
       </c>
       <c r="J801" t="inlineStr">
         <is>
-          <t>BORGERS USA CORP</t>
+          <t>VISUAL CREATIONS, INC.</t>
         </is>
       </c>
       <c r="K801" t="inlineStr">
         <is>
-          <t>BORUSA</t>
+          <t>VISCRE</t>
         </is>
       </c>
       <c r="L801" t="inlineStr">
         <is>
-          <t>65-117296500</t>
+          <t>20-461602300</t>
         </is>
       </c>
       <c r="M801" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="N801" t="inlineStr">
         <is>
-          <t>2026-07-02 00:00:00</t>
+          <t>2026-07-04 00:00:00</t>
         </is>
       </c>
       <c r="O801" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="P801" t="inlineStr">
         <is>
-          <t>AUTONEUM CZ S.R.O.</t>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
         </is>
       </c>
       <c r="Q801" t="inlineStr">
         <is>
-          <t>2026-06-20 00:00:00</t>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2566192</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>EF4-0232351-5</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr"/>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>1108.14.0000</t>
+        </is>
+      </c>
+      <c r="J802" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K802" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L802" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M802" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N802" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="O802" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="P802" t="inlineStr">
+        <is>
+          <t>SANGUAN WONGSE STARCH CO., LTD.</t>
+        </is>
+      </c>
+      <c r="Q802" t="inlineStr">
+        <is>
+          <t>2026-06-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2566349</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>EF4-0232573-4</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr"/>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr"/>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>1108.12.0010</t>
+        </is>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K803" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L803" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M803" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N803" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="O803" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="P803" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="Q803" t="inlineStr">
+        <is>
+          <t>2026-06-13 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2566272</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>EF4-0232670-8</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>V1626472883</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>1702.30.4085</t>
+        </is>
+      </c>
+      <c r="J804" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K804" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L804" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M804" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N804" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="O804" t="inlineStr">
+        <is>
+          <t>AK NISASTA SANAYI VE TICARET AS</t>
+        </is>
+      </c>
+      <c r="P804" t="inlineStr">
+        <is>
+          <t>AK NISASTA SANAYI VE TICARET AS</t>
+        </is>
+      </c>
+      <c r="Q804" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append trimika data — 24 new rows, 827 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q804"/>
+  <dimension ref="A1:Q828"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67656,6 +67656,2018 @@
         </is>
       </c>
     </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2565992</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>EF4-0232152-7</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr"/>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J805" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K805" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L805" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M805" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N805" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O805" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P805" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q805" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2566077</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>EF4-0232194-9</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr"/>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J806" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K806" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L806" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M806" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N806" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O806" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P806" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q806" t="inlineStr">
+        <is>
+          <t>2026-05-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2566118</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>EF4-0232255-8</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr"/>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8302.42.3065</t>
+        </is>
+      </c>
+      <c r="J807" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K807" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L807" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M807" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N807" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O807" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P807" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q807" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2566118</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>EF4-0232255-8</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr"/>
+      <c r="E808" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F808" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I808" t="inlineStr">
+        <is>
+          <t>9903.03.01,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J808" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K808" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L808" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M808" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N808" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O808" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P808" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q808" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2566118</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>EF4-0232255-8</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr"/>
+      <c r="E809" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F809" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I809" t="inlineStr">
+        <is>
+          <t>9903.03.01,9903.76.04,9403.91.0080</t>
+        </is>
+      </c>
+      <c r="J809" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K809" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L809" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M809" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N809" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O809" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P809" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q809" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr"/>
+      <c r="E810" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F810" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I810" t="inlineStr">
+        <is>
+          <t>9903.03.01,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J810" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K810" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L810" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M810" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N810" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O810" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P810" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q810" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr"/>
+      <c r="E811" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F811" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I811" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.02,7318.19.0000</t>
+        </is>
+      </c>
+      <c r="J811" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K811" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L811" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M811" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N811" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O811" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P811" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q811" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr"/>
+      <c r="E812" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F812" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I812" t="inlineStr">
+        <is>
+          <t>9903.03.01,9405.42.8440</t>
+        </is>
+      </c>
+      <c r="J812" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K812" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L812" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M812" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N812" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O812" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P812" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q812" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr"/>
+      <c r="E813" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F813" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I813" t="inlineStr">
+        <is>
+          <t>9903.03.01,9903.76.04,9403.60.8093</t>
+        </is>
+      </c>
+      <c r="J813" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K813" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L813" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M813" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N813" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O813" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P813" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q813" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr"/>
+      <c r="E814" t="inlineStr">
+        <is>
+          <t>9903.88.02</t>
+        </is>
+      </c>
+      <c r="F814" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(C)</t>
+        </is>
+      </c>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>9903.88.02</t>
+        </is>
+      </c>
+      <c r="I814" t="inlineStr">
+        <is>
+          <t>9903.03.01,8536.30.8000</t>
+        </is>
+      </c>
+      <c r="J814" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K814" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L814" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M814" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N814" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O814" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P814" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q814" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr"/>
+      <c r="E815" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F815" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I815" t="inlineStr">
+        <is>
+          <t>9903.03.01,3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J815" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K815" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L815" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M815" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N815" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O815" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P815" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q815" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr"/>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F816" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>9903.03.01,9405.41.8440</t>
+        </is>
+      </c>
+      <c r="J816" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K816" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L816" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M816" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N816" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O816" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P816" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q816" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr"/>
+      <c r="E817" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="F817" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(R)</t>
+        </is>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>9903.88.15</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,8302.42.3065</t>
+        </is>
+      </c>
+      <c r="J817" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K817" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L817" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M817" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N817" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O817" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P817" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q817" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2566127</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>EF4-0232257-4</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr"/>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F818" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I818" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.82.09,9403.20.0075</t>
+        </is>
+      </c>
+      <c r="J818" t="inlineStr">
+        <is>
+          <t>VISUAL CREATIONS, INC.</t>
+        </is>
+      </c>
+      <c r="K818" t="inlineStr">
+        <is>
+          <t>VISCRE</t>
+        </is>
+      </c>
+      <c r="L818" t="inlineStr">
+        <is>
+          <t>20-461602300</t>
+        </is>
+      </c>
+      <c r="M818" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N818" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O818" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="P818" t="inlineStr">
+        <is>
+          <t>FUJIAN ANTAI NEW ENERGY TECH CO LTD</t>
+        </is>
+      </c>
+      <c r="Q818" t="inlineStr">
+        <is>
+          <t>2026-05-31 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2566098</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>EF4-0232438-0</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr"/>
+      <c r="E819" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F819" t="inlineStr"/>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I819" t="inlineStr">
+        <is>
+          <t>1108.12.0010</t>
+        </is>
+      </c>
+      <c r="J819" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K819" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L819" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M819" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N819" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O819" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="P819" t="inlineStr">
+        <is>
+          <t>TAT NISASTA INS SAN TIC AS</t>
+        </is>
+      </c>
+      <c r="Q819" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2566326</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>EF4-0232459-6</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr"/>
+      <c r="E820" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F820" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I820" t="inlineStr">
+        <is>
+          <t>4409.29.0655</t>
+        </is>
+      </c>
+      <c r="J820" t="inlineStr">
+        <is>
+          <t>AUTHENTIC SURFACES LLC</t>
+        </is>
+      </c>
+      <c r="K820" t="inlineStr">
+        <is>
+          <t>AUTSUR01</t>
+        </is>
+      </c>
+      <c r="L820" t="inlineStr">
+        <is>
+          <t>86-279678900</t>
+        </is>
+      </c>
+      <c r="M820" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N820" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O820" t="inlineStr">
+        <is>
+          <t>CHENE DE L'EST</t>
+        </is>
+      </c>
+      <c r="P820" t="inlineStr">
+        <is>
+          <t>CHENE DE L'EST</t>
+        </is>
+      </c>
+      <c r="Q820" t="inlineStr">
+        <is>
+          <t>2026-06-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2566274</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>EF4-0232541-1</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>V1626485778</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F821" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I821" t="inlineStr">
+        <is>
+          <t>1702.30.4085</t>
+        </is>
+      </c>
+      <c r="J821" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K821" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L821" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M821" t="inlineStr">
+        <is>
+          <t>2026-07-01 00:00:00</t>
+        </is>
+      </c>
+      <c r="N821" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O821" t="inlineStr">
+        <is>
+          <t>AK NISASTA SANAYI VE TICARET AS</t>
+        </is>
+      </c>
+      <c r="P821" t="inlineStr">
+        <is>
+          <t>AK NISASTA SANAYI VE TICARET AS</t>
+        </is>
+      </c>
+      <c r="Q821" t="inlineStr">
+        <is>
+          <t>2026-06-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2566271</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>EF4-0232613-8</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>V1626485778</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F822" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>9903.82.22,8427.90.0090</t>
+        </is>
+      </c>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K822" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L822" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M822" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N822" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O822" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P822" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q822" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2566271</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>EF4-0232613-8</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>V1626485778</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F823" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>9903.82.22,8427.90.0090</t>
+        </is>
+      </c>
+      <c r="J823" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K823" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L823" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M823" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N823" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O823" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P823" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q823" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2566271</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>EF4-0232613-8</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>V1626485778</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F824" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I824" t="inlineStr">
+        <is>
+          <t>9903.82.22,8427.90.0090</t>
+        </is>
+      </c>
+      <c r="J824" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K824" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L824" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M824" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N824" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O824" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P824" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q824" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2566271</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>EF4-0232613-8</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>V1626485778</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F825" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I825" t="inlineStr">
+        <is>
+          <t>9903.82.22,8427.90.0090</t>
+        </is>
+      </c>
+      <c r="J825" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K825" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L825" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M825" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N825" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O825" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P825" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q825" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2566271</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>EF4-0232613-8</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>V1626485778</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F826" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I826" t="inlineStr">
+        <is>
+          <t>9903.82.22,8427.90.0090</t>
+        </is>
+      </c>
+      <c r="J826" t="inlineStr">
+        <is>
+          <t>MALLAGHAN (GA) INC.</t>
+        </is>
+      </c>
+      <c r="K826" t="inlineStr">
+        <is>
+          <t>MALGA01</t>
+        </is>
+      </c>
+      <c r="L826" t="inlineStr">
+        <is>
+          <t>36-488102800</t>
+        </is>
+      </c>
+      <c r="M826" t="inlineStr">
+        <is>
+          <t>2026-07-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="N826" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O826" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="P826" t="inlineStr">
+        <is>
+          <t>MALLAGHAN ENGINEERING  LTD</t>
+        </is>
+      </c>
+      <c r="Q826" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>105504864</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>EF4-0232978-5</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr"/>
+      <c r="E827" t="inlineStr">
+        <is>
+          <t>9817.85.01</t>
+        </is>
+      </c>
+      <c r="F827" t="inlineStr">
+        <is>
+          <t>PROTOTYPES, TESTING/EVALUATION</t>
+        </is>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>9817.85.01</t>
+        </is>
+      </c>
+      <c r="I827" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.94.51,8703.23.0160</t>
+        </is>
+      </c>
+      <c r="J827" t="inlineStr">
+        <is>
+          <t>PORSCHE MOTORSPORT NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K827" t="inlineStr">
+        <is>
+          <t>PORMOT01</t>
+        </is>
+      </c>
+      <c r="L827" t="inlineStr">
+        <is>
+          <t>23-234420600</t>
+        </is>
+      </c>
+      <c r="M827" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N827" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O827" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN SLOVAKIA A.S</t>
+        </is>
+      </c>
+      <c r="P827" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN SLOVAKIA A.S</t>
+        </is>
+      </c>
+      <c r="Q827" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>105504866</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>EF4-0232983-5</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr"/>
+      <c r="E828" t="inlineStr">
+        <is>
+          <t>9817.85.01</t>
+        </is>
+      </c>
+      <c r="F828" t="inlineStr">
+        <is>
+          <t>PROTOTYPES, TESTING/EVALUATION</t>
+        </is>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>9817.85.01</t>
+        </is>
+      </c>
+      <c r="I828" t="inlineStr">
+        <is>
+          <t>9903.03.06,9903.94.51,8703.60.0030</t>
+        </is>
+      </c>
+      <c r="J828" t="inlineStr">
+        <is>
+          <t>PORSCHE MOTORSPORT NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K828" t="inlineStr">
+        <is>
+          <t>PORMOT01</t>
+        </is>
+      </c>
+      <c r="L828" t="inlineStr">
+        <is>
+          <t>23-234420600</t>
+        </is>
+      </c>
+      <c r="M828" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N828" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="O828" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN SLOVAKIA A.S</t>
+        </is>
+      </c>
+      <c r="P828" t="inlineStr">
+        <is>
+          <t>VOLKSWAGEN SLOVAKIA A.S</t>
+        </is>
+      </c>
+      <c r="Q828" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 31 new rows, 858 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q828"/>
+  <dimension ref="A1:Q859"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69668,6 +69668,2667 @@
         </is>
       </c>
     </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2565921</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>EF4-0231891-1</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>165925675</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>9803.00.50</t>
+        </is>
+      </c>
+      <c r="F829" t="inlineStr">
+        <is>
+          <t>SUBSTANTIAL CONTAINERS US&amp;INTL</t>
+        </is>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>9803.00.50</t>
+        </is>
+      </c>
+      <c r="I829" t="inlineStr"/>
+      <c r="J829" t="inlineStr">
+        <is>
+          <t>MEBROM LLC</t>
+        </is>
+      </c>
+      <c r="K829" t="inlineStr">
+        <is>
+          <t>MEBLLC01</t>
+        </is>
+      </c>
+      <c r="L829" t="inlineStr">
+        <is>
+          <t>84-463527000</t>
+        </is>
+      </c>
+      <c r="M829" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N829" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O829" t="inlineStr">
+        <is>
+          <t>SAHAMITR PRESSURE CONTAINER PUBLIC</t>
+        </is>
+      </c>
+      <c r="P829" t="inlineStr">
+        <is>
+          <t>SAHAMITR PRESSURE CONTAINER PUBLIC CO LTD</t>
+        </is>
+      </c>
+      <c r="Q829" t="inlineStr">
+        <is>
+          <t>2026-05-15 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2565904</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>EF4-0231900-0</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr"/>
+      <c r="E830" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F830" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I830" t="inlineStr">
+        <is>
+          <t>5603.14.9090</t>
+        </is>
+      </c>
+      <c r="J830" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K830" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L830" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M830" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N830" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O830" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P830" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q830" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2565991</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>EF4-0231968-7</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr"/>
+      <c r="E831" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F831" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I831" t="inlineStr">
+        <is>
+          <t>5603.14.9090</t>
+        </is>
+      </c>
+      <c r="J831" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K831" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L831" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M831" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N831" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O831" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P831" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q831" t="inlineStr">
+        <is>
+          <t>2026-05-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2566335</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>EF4-0232734-2</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr"/>
+      <c r="E832" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F832" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I832" t="inlineStr">
+        <is>
+          <t>3920.20.0055</t>
+        </is>
+      </c>
+      <c r="J832" t="inlineStr">
+        <is>
+          <t>TEUFELBERGER G.E.S.M.B.H</t>
+        </is>
+      </c>
+      <c r="K832" t="inlineStr">
+        <is>
+          <t>TEUSEI01</t>
+        </is>
+      </c>
+      <c r="L832" t="inlineStr">
+        <is>
+          <t>181704-13780</t>
+        </is>
+      </c>
+      <c r="M832" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N832" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O832" t="inlineStr">
+        <is>
+          <t>TEUFELBERGER GMBH</t>
+        </is>
+      </c>
+      <c r="P832" t="inlineStr">
+        <is>
+          <t>TEUFELBERGER GMBH</t>
+        </is>
+      </c>
+      <c r="Q832" t="inlineStr">
+        <is>
+          <t>2026-06-16 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F833" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I833" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J833" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K833" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L833" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M833" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N833" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O833" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P833" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q833" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F834" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I834" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J834" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K834" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L834" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M834" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N834" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O834" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P834" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q834" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F835" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I835" t="inlineStr">
+        <is>
+          <t>9903.82.09,8483.10.5000</t>
+        </is>
+      </c>
+      <c r="J835" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K835" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L835" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M835" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N835" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O835" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P835" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q835" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F836" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I836" t="inlineStr">
+        <is>
+          <t>9903.82.09,8483.10.5000</t>
+        </is>
+      </c>
+      <c r="J836" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K836" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L836" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M836" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N836" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O836" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P836" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q836" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F837" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I837" t="inlineStr">
+        <is>
+          <t>9903.82.09,8483.10.5000</t>
+        </is>
+      </c>
+      <c r="J837" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K837" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L837" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M837" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N837" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O837" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P837" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q837" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F838" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I838" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J838" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K838" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L838" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M838" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N838" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O838" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P838" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q838" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F839" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I839" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J839" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K839" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L839" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M839" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N839" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O839" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P839" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q839" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F840" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I840" t="inlineStr">
+        <is>
+          <t>9903.82.01,8483.30.8040</t>
+        </is>
+      </c>
+      <c r="J840" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K840" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L840" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M840" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N840" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O840" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P840" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q840" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F841" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I841" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J841" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K841" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L841" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M841" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N841" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O841" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P841" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q841" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F842" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I842" t="inlineStr">
+        <is>
+          <t>8481.80.3075</t>
+        </is>
+      </c>
+      <c r="J842" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K842" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L842" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M842" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N842" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O842" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P842" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q842" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F843" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I843" t="inlineStr">
+        <is>
+          <t>8481.80.3075</t>
+        </is>
+      </c>
+      <c r="J843" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K843" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L843" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M843" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N843" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O843" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P843" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q843" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F844" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I844" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J844" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K844" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L844" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M844" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N844" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O844" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P844" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q844" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F845" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I845" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J845" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K845" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L845" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M845" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N845" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O845" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P845" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q845" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F846" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J846" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K846" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L846" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M846" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N846" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O846" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P846" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q846" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F847" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I847" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J847" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K847" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L847" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M847" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N847" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O847" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P847" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q847" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I848" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J848" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K848" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L848" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M848" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N848" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O848" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P848" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q848" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I849" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J849" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K849" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L849" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M849" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N849" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O849" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P849" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q849" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>4539551</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>EF4-0232798-7</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I850" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J850" t="inlineStr">
+        <is>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+        </is>
+      </c>
+      <c r="K850" t="inlineStr">
+        <is>
+          <t>EISINC03</t>
+        </is>
+      </c>
+      <c r="L850" t="inlineStr">
+        <is>
+          <t>86-240963300</t>
+        </is>
+      </c>
+      <c r="M850" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N850" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O850" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="P850" t="inlineStr">
+        <is>
+          <t>EISENMANN GMBH</t>
+        </is>
+      </c>
+      <c r="Q850" t="inlineStr">
+        <is>
+          <t>2026-06-27 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2566499</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>EF4-0232832-4</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I851" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J851" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K851" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L851" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M851" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N851" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O851" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+        </is>
+      </c>
+      <c r="P851" t="inlineStr">
+        <is>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+        </is>
+      </c>
+      <c r="Q851" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2566276</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>EF4-0232875-3</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>V0710334835</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I852" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1061</t>
+        </is>
+      </c>
+      <c r="J852" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K852" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L852" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M852" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N852" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O852" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
+        </is>
+      </c>
+      <c r="P852" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="Q852" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2566298</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>EF4-0232877-9</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>V0710334835</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I853" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1061</t>
+        </is>
+      </c>
+      <c r="J853" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="K853" t="inlineStr">
+        <is>
+          <t>PREMET</t>
+        </is>
+      </c>
+      <c r="L853" t="inlineStr">
+        <is>
+          <t>172704-21182</t>
+        </is>
+      </c>
+      <c r="M853" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N853" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O853" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P853" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q853" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2566298</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>EF4-0232877-9</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>V0710334835</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I854" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1076</t>
+        </is>
+      </c>
+      <c r="J854" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="K854" t="inlineStr">
+        <is>
+          <t>PREMET</t>
+        </is>
+      </c>
+      <c r="L854" t="inlineStr">
+        <is>
+          <t>172704-21182</t>
+        </is>
+      </c>
+      <c r="M854" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N854" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O854" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P854" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q854" t="inlineStr">
+        <is>
+          <t>2026-06-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>4539589</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>EF4-0232907-4</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr"/>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I855" t="inlineStr">
+        <is>
+          <t>3926.30.5000</t>
+        </is>
+      </c>
+      <c r="J855" t="inlineStr">
+        <is>
+          <t>NOLTE USA LLC</t>
+        </is>
+      </c>
+      <c r="K855" t="inlineStr">
+        <is>
+          <t>NOLUSA01</t>
+        </is>
+      </c>
+      <c r="L855" t="inlineStr">
+        <is>
+          <t>46-224248300</t>
+        </is>
+      </c>
+      <c r="M855" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N855" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O855" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="P855" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="Q855" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>4539589</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>EF4-0232907-4</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr"/>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I856" t="inlineStr">
+        <is>
+          <t>9903.82.09,8302.42.3065</t>
+        </is>
+      </c>
+      <c r="J856" t="inlineStr">
+        <is>
+          <t>NOLTE USA LLC</t>
+        </is>
+      </c>
+      <c r="K856" t="inlineStr">
+        <is>
+          <t>NOLUSA01</t>
+        </is>
+      </c>
+      <c r="L856" t="inlineStr">
+        <is>
+          <t>46-224248300</t>
+        </is>
+      </c>
+      <c r="M856" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N856" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O856" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="P856" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="Q856" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>4539589</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>EF4-0232907-4</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr"/>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I857" t="inlineStr">
+        <is>
+          <t>9903.82.09,9403.99.9045</t>
+        </is>
+      </c>
+      <c r="J857" t="inlineStr">
+        <is>
+          <t>NOLTE USA LLC</t>
+        </is>
+      </c>
+      <c r="K857" t="inlineStr">
+        <is>
+          <t>NOLUSA01</t>
+        </is>
+      </c>
+      <c r="L857" t="inlineStr">
+        <is>
+          <t>46-224248300</t>
+        </is>
+      </c>
+      <c r="M857" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N857" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O857" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="P857" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="Q857" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>4539589</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>EF4-0232907-4</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr"/>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I858" t="inlineStr">
+        <is>
+          <t>9903.76.22,9403.40.9060</t>
+        </is>
+      </c>
+      <c r="J858" t="inlineStr">
+        <is>
+          <t>NOLTE USA LLC</t>
+        </is>
+      </c>
+      <c r="K858" t="inlineStr">
+        <is>
+          <t>NOLUSA01</t>
+        </is>
+      </c>
+      <c r="L858" t="inlineStr">
+        <is>
+          <t>46-224248300</t>
+        </is>
+      </c>
+      <c r="M858" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N858" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O858" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="P858" t="inlineStr">
+        <is>
+          <t>NOLTE KUCHEN GMBH</t>
+        </is>
+      </c>
+      <c r="Q858" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>4539623</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>EF4-0233010-6</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr"/>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.06,8537.10.9170</t>
+        </is>
+      </c>
+      <c r="J859" t="inlineStr">
+        <is>
+          <t>QUANTUM TECHNOLOGY SYSTEMS LLC</t>
+        </is>
+      </c>
+      <c r="K859" t="inlineStr">
+        <is>
+          <t>QUATEC01</t>
+        </is>
+      </c>
+      <c r="L859" t="inlineStr">
+        <is>
+          <t>33-167928800</t>
+        </is>
+      </c>
+      <c r="M859" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N859" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="O859" t="inlineStr">
+        <is>
+          <t>ELCOM INTERNATIONAL PVT LTD</t>
+        </is>
+      </c>
+      <c r="P859" t="inlineStr">
+        <is>
+          <t>ELCOM INTERNATIONAL PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q859" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 41 new rows, 898 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q859"/>
+  <dimension ref="A1:Q899"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69754,12 +69754,12 @@
     <row r="830">
       <c r="A830" t="inlineStr">
         <is>
-          <t>2565904</t>
+          <t>2565991</t>
         </is>
       </c>
       <c r="B830" t="inlineStr">
         <is>
-          <t>EF4-0231900-0</t>
+          <t>EF4-0231968-7</t>
         </is>
       </c>
       <c r="C830" t="inlineStr">
@@ -69810,7 +69810,7 @@
       </c>
       <c r="M830" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-07 00:00:00</t>
         </is>
       </c>
       <c r="N830" t="inlineStr">
@@ -69830,19 +69830,19 @@
       </c>
       <c r="Q830" t="inlineStr">
         <is>
-          <t>2026-05-12 00:00:00</t>
+          <t>2026-05-19 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr">
         <is>
-          <t>2565991</t>
+          <t>2566335</t>
         </is>
       </c>
       <c r="B831" t="inlineStr">
         <is>
-          <t>EF4-0231968-7</t>
+          <t>EF4-0232734-2</t>
         </is>
       </c>
       <c r="C831" t="inlineStr">
@@ -69873,22 +69873,22 @@
       </c>
       <c r="I831" t="inlineStr">
         <is>
-          <t>5603.14.9090</t>
+          <t>3920.20.0055</t>
         </is>
       </c>
       <c r="J831" t="inlineStr">
         <is>
-          <t>VEER CORPORATIONS INC</t>
+          <t>TEUFELBERGER G.E.S.M.B.H</t>
         </is>
       </c>
       <c r="K831" t="inlineStr">
         <is>
-          <t>VEECOR01</t>
+          <t>TEUSEI01</t>
         </is>
       </c>
       <c r="L831" t="inlineStr">
         <is>
-          <t>99-106989200</t>
+          <t>181704-13780</t>
         </is>
       </c>
       <c r="M831" t="inlineStr">
@@ -69903,45 +69903,49 @@
       </c>
       <c r="O831" t="inlineStr">
         <is>
-          <t>VEER PLASTIC PVT LTD</t>
+          <t>TEUFELBERGER GMBH</t>
         </is>
       </c>
       <c r="P831" t="inlineStr">
         <is>
-          <t>VEER PLASTIC PVT LTD</t>
+          <t>TEUFELBERGER GMBH</t>
         </is>
       </c>
       <c r="Q831" t="inlineStr">
         <is>
-          <t>2026-05-19 00:00:00</t>
+          <t>2026-06-16 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr">
         <is>
-          <t>2566335</t>
+          <t>4539551</t>
         </is>
       </c>
       <c r="B832" t="inlineStr">
         <is>
-          <t>EF4-0232734-2</t>
+          <t>EF4-0232798-7</t>
         </is>
       </c>
       <c r="C832" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
-        </is>
-      </c>
-      <c r="D832" t="inlineStr"/>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>02031887483</t>
+        </is>
+      </c>
       <c r="E832" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F832" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G832" t="inlineStr">
@@ -69951,52 +69955,52 @@
       </c>
       <c r="H832" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I832" t="inlineStr">
         <is>
-          <t>3920.20.0055</t>
+          <t>9903.82.10,8431.39.0010</t>
         </is>
       </c>
       <c r="J832" t="inlineStr">
         <is>
-          <t>TEUFELBERGER G.E.S.M.B.H</t>
+          <t>EISENMANN OF SOUTH CAROLINA INC</t>
         </is>
       </c>
       <c r="K832" t="inlineStr">
         <is>
-          <t>TEUSEI01</t>
+          <t>EISINC03</t>
         </is>
       </c>
       <c r="L832" t="inlineStr">
         <is>
-          <t>181704-13780</t>
+          <t>86-240963300</t>
         </is>
       </c>
       <c r="M832" t="inlineStr">
         <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N832" t="inlineStr">
+        <is>
           <t>2026-07-07 00:00:00</t>
         </is>
       </c>
-      <c r="N832" t="inlineStr">
-        <is>
-          <t>2026-07-07 00:00:00</t>
-        </is>
-      </c>
       <c r="O832" t="inlineStr">
         <is>
-          <t>TEUFELBERGER GMBH</t>
+          <t>EISENMANN GMBH</t>
         </is>
       </c>
       <c r="P832" t="inlineStr">
         <is>
-          <t>TEUFELBERGER GMBH</t>
+          <t>EISENMANN GMBH</t>
         </is>
       </c>
       <c r="Q832" t="inlineStr">
         <is>
-          <t>2026-06-16 00:00:00</t>
+          <t>2026-06-27 00:00:00</t>
         </is>
       </c>
     </row>
@@ -70033,7 +70037,7 @@
       </c>
       <c r="G833" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H833" t="inlineStr">
@@ -70120,7 +70124,7 @@
       </c>
       <c r="G834" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H834" t="inlineStr">
@@ -70130,7 +70134,7 @@
       </c>
       <c r="I834" t="inlineStr">
         <is>
-          <t>9903.82.10,8431.39.0010</t>
+          <t>9903.82.09,8483.10.5000</t>
         </is>
       </c>
       <c r="J834" t="inlineStr">
@@ -70207,7 +70211,7 @@
       </c>
       <c r="G835" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H835" t="inlineStr">
@@ -70294,7 +70298,7 @@
       </c>
       <c r="G836" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>005</t>
         </is>
       </c>
       <c r="H836" t="inlineStr">
@@ -70381,7 +70385,7 @@
       </c>
       <c r="G837" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>006</t>
         </is>
       </c>
       <c r="H837" t="inlineStr">
@@ -70391,7 +70395,7 @@
       </c>
       <c r="I837" t="inlineStr">
         <is>
-          <t>9903.82.09,8483.10.5000</t>
+          <t>9903.82.10,8431.39.0010</t>
         </is>
       </c>
       <c r="J837" t="inlineStr">
@@ -70468,7 +70472,7 @@
       </c>
       <c r="G838" t="inlineStr">
         <is>
-          <t>006</t>
+          <t>007</t>
         </is>
       </c>
       <c r="H838" t="inlineStr">
@@ -70545,27 +70549,27 @@
       </c>
       <c r="E839" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F839" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G839" t="inlineStr">
         <is>
-          <t>007</t>
+          <t>008</t>
         </is>
       </c>
       <c r="H839" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I839" t="inlineStr">
         <is>
-          <t>9903.82.10,8431.39.0010</t>
+          <t>9903.82.01,8483.30.8040</t>
         </is>
       </c>
       <c r="J839" t="inlineStr">
@@ -70632,27 +70636,27 @@
       </c>
       <c r="E840" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F840" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G840" t="inlineStr">
         <is>
-          <t>008</t>
+          <t>009</t>
         </is>
       </c>
       <c r="H840" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I840" t="inlineStr">
         <is>
-          <t>9903.82.01,8483.30.8040</t>
+          <t>9903.82.10,8431.39.0010</t>
         </is>
       </c>
       <c r="J840" t="inlineStr">
@@ -70719,27 +70723,27 @@
       </c>
       <c r="E841" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F841" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G841" t="inlineStr">
         <is>
-          <t>009</t>
+          <t>010</t>
         </is>
       </c>
       <c r="H841" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I841" t="inlineStr">
         <is>
-          <t>9903.82.10,8431.39.0010</t>
+          <t>8481.80.3075</t>
         </is>
       </c>
       <c r="J841" t="inlineStr">
@@ -70816,7 +70820,7 @@
       </c>
       <c r="G842" t="inlineStr">
         <is>
-          <t>010</t>
+          <t>011</t>
         </is>
       </c>
       <c r="H842" t="inlineStr">
@@ -70893,27 +70897,27 @@
       </c>
       <c r="E843" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F843" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G843" t="inlineStr">
         <is>
-          <t>011</t>
+          <t>012</t>
         </is>
       </c>
       <c r="H843" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I843" t="inlineStr">
         <is>
-          <t>8481.80.3075</t>
+          <t>9903.82.10,8431.39.0010</t>
         </is>
       </c>
       <c r="J843" t="inlineStr">
@@ -70990,7 +70994,7 @@
       </c>
       <c r="G844" t="inlineStr">
         <is>
-          <t>012</t>
+          <t>013</t>
         </is>
       </c>
       <c r="H844" t="inlineStr">
@@ -71077,7 +71081,7 @@
       </c>
       <c r="G845" t="inlineStr">
         <is>
-          <t>013</t>
+          <t>014</t>
         </is>
       </c>
       <c r="H845" t="inlineStr">
@@ -71164,7 +71168,7 @@
       </c>
       <c r="G846" t="inlineStr">
         <is>
-          <t>014</t>
+          <t>015</t>
         </is>
       </c>
       <c r="H846" t="inlineStr">
@@ -71251,7 +71255,7 @@
       </c>
       <c r="G847" t="inlineStr">
         <is>
-          <t>015</t>
+          <t>016</t>
         </is>
       </c>
       <c r="H847" t="inlineStr">
@@ -71338,7 +71342,7 @@
       </c>
       <c r="G848" t="inlineStr">
         <is>
-          <t>016</t>
+          <t>017</t>
         </is>
       </c>
       <c r="H848" t="inlineStr">
@@ -71425,7 +71429,7 @@
       </c>
       <c r="G849" t="inlineStr">
         <is>
-          <t>017</t>
+          <t>018</t>
         </is>
       </c>
       <c r="H849" t="inlineStr">
@@ -71482,17 +71486,17 @@
     <row r="850">
       <c r="A850" t="inlineStr">
         <is>
-          <t>4539551</t>
+          <t>2566499</t>
         </is>
       </c>
       <c r="B850" t="inlineStr">
         <is>
-          <t>EF4-0232798-7</t>
+          <t>EF4-0232832-4</t>
         </is>
       </c>
       <c r="C850" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D850" t="inlineStr">
@@ -71502,47 +71506,47 @@
       </c>
       <c r="E850" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F850" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G850" t="inlineStr">
         <is>
-          <t>018</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H850" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I850" t="inlineStr">
         <is>
-          <t>9903.82.10,8431.39.0010</t>
+          <t>1109.00.9020</t>
         </is>
       </c>
       <c r="J850" t="inlineStr">
         <is>
-          <t>EISENMANN OF SOUTH CAROLINA INC</t>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
         </is>
       </c>
       <c r="K850" t="inlineStr">
         <is>
-          <t>EISINC03</t>
+          <t>ROYINGRE</t>
         </is>
       </c>
       <c r="L850" t="inlineStr">
         <is>
-          <t>86-240963300</t>
+          <t>074601-00962</t>
         </is>
       </c>
       <c r="M850" t="inlineStr">
         <is>
-          <t>2026-07-03 00:00:00</t>
+          <t>2026-07-07 00:00:00</t>
         </is>
       </c>
       <c r="N850" t="inlineStr">
@@ -71552,29 +71556,29 @@
       </c>
       <c r="O850" t="inlineStr">
         <is>
-          <t>EISENMANN GMBH</t>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
         </is>
       </c>
       <c r="P850" t="inlineStr">
         <is>
-          <t>EISENMANN GMBH</t>
+          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
         </is>
       </c>
       <c r="Q850" t="inlineStr">
         <is>
-          <t>2026-06-27 00:00:00</t>
+          <t>2026-06-25 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="851">
       <c r="A851" t="inlineStr">
         <is>
-          <t>2566499</t>
+          <t>2566276</t>
         </is>
       </c>
       <c r="B851" t="inlineStr">
         <is>
-          <t>EF4-0232832-4</t>
+          <t>EF4-0232875-3</t>
         </is>
       </c>
       <c r="C851" t="inlineStr">
@@ -71584,17 +71588,17 @@
       </c>
       <c r="D851" t="inlineStr">
         <is>
-          <t>02031887483</t>
+          <t>V0710334835</t>
         </is>
       </c>
       <c r="E851" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F851" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G851" t="inlineStr">
@@ -71604,27 +71608,27 @@
       </c>
       <c r="H851" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I851" t="inlineStr">
         <is>
-          <t>1109.00.9020</t>
+          <t>9903.82.02,7223.00.1061</t>
         </is>
       </c>
       <c r="J851" t="inlineStr">
         <is>
-          <t>ROYAL INGREDIENTS GROUP BV</t>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
         </is>
       </c>
       <c r="K851" t="inlineStr">
         <is>
-          <t>ROYINGRE</t>
+          <t>VENWIR</t>
         </is>
       </c>
       <c r="L851" t="inlineStr">
         <is>
-          <t>074601-00962</t>
+          <t>993901-03595</t>
         </is>
       </c>
       <c r="M851" t="inlineStr">
@@ -71639,29 +71643,29 @@
       </c>
       <c r="O851" t="inlineStr">
         <is>
-          <t>JACKERING MUHLEN UND NAHRMITTELWERK</t>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
         </is>
       </c>
       <c r="P851" t="inlineStr">
         <is>
-          <t>JACKERING MUHLEN UND NAHRMITTELWERKE GMBH</t>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
         </is>
       </c>
       <c r="Q851" t="inlineStr">
         <is>
-          <t>2026-06-25 00:00:00</t>
+          <t>2026-06-06 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
         <is>
-          <t>2566276</t>
+          <t>2566298</t>
         </is>
       </c>
       <c r="B852" t="inlineStr">
         <is>
-          <t>EF4-0232875-3</t>
+          <t>EF4-0232877-9</t>
         </is>
       </c>
       <c r="C852" t="inlineStr">
@@ -71701,17 +71705,17 @@
       </c>
       <c r="J852" t="inlineStr">
         <is>
-          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+          <t>PRECISION METALS</t>
         </is>
       </c>
       <c r="K852" t="inlineStr">
         <is>
-          <t>VENWIR</t>
+          <t>PREMET</t>
         </is>
       </c>
       <c r="L852" t="inlineStr">
         <is>
-          <t>993901-03595</t>
+          <t>172704-21182</t>
         </is>
       </c>
       <c r="M852" t="inlineStr">
@@ -71726,12 +71730,12 @@
       </c>
       <c r="O852" t="inlineStr">
         <is>
-          <t>VENUS WIRE INDUSTRIES PRIVATE LIMIT</t>
+          <t>PRECISION METALS</t>
         </is>
       </c>
       <c r="P852" t="inlineStr">
         <is>
-          <t>VENUS WIRE INDUSTRIES PRIVATE LIMITED</t>
+          <t>PRECISION METALS</t>
         </is>
       </c>
       <c r="Q852" t="inlineStr">
@@ -71773,7 +71777,7 @@
       </c>
       <c r="G853" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H853" t="inlineStr">
@@ -71783,7 +71787,7 @@
       </c>
       <c r="I853" t="inlineStr">
         <is>
-          <t>9903.82.02,7223.00.1061</t>
+          <t>9903.82.02,7223.00.1076</t>
         </is>
       </c>
       <c r="J853" t="inlineStr">
@@ -71830,87 +71834,83 @@
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t>2566298</t>
+          <t>4539589</t>
         </is>
       </c>
       <c r="B854" t="inlineStr">
         <is>
-          <t>EF4-0232877-9</t>
+          <t>EF4-0232907-4</t>
         </is>
       </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>Vessel, Container</t>
-        </is>
-      </c>
-      <c r="D854" t="inlineStr">
-        <is>
-          <t>V0710334835</t>
-        </is>
-      </c>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr"/>
       <c r="E854" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F854" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G854" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H854" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I854" t="inlineStr">
         <is>
-          <t>9903.82.02,7223.00.1076</t>
+          <t>3926.30.5000</t>
         </is>
       </c>
       <c r="J854" t="inlineStr">
         <is>
-          <t>PRECISION METALS</t>
+          <t>NOLTE USA LLC</t>
         </is>
       </c>
       <c r="K854" t="inlineStr">
         <is>
-          <t>PREMET</t>
+          <t>NOLUSA01</t>
         </is>
       </c>
       <c r="L854" t="inlineStr">
         <is>
-          <t>172704-21182</t>
+          <t>46-224248300</t>
         </is>
       </c>
       <c r="M854" t="inlineStr">
         <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N854" t="inlineStr">
+        <is>
           <t>2026-07-07 00:00:00</t>
         </is>
       </c>
-      <c r="N854" t="inlineStr">
-        <is>
-          <t>2026-07-07 00:00:00</t>
-        </is>
-      </c>
       <c r="O854" t="inlineStr">
         <is>
-          <t>PRECISION METALS</t>
+          <t>NOLTE KUCHEN GMBH</t>
         </is>
       </c>
       <c r="P854" t="inlineStr">
         <is>
-          <t>PRECISION METALS</t>
+          <t>NOLTE KUCHEN GMBH</t>
         </is>
       </c>
       <c r="Q854" t="inlineStr">
         <is>
-          <t>2026-06-06 00:00:00</t>
+          <t>2026-07-06 00:00:00</t>
         </is>
       </c>
     </row>
@@ -71933,27 +71933,27 @@
       <c r="D855" t="inlineStr"/>
       <c r="E855" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F855" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G855" t="inlineStr">
         <is>
-          <t>001</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H855" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I855" t="inlineStr">
         <is>
-          <t>3926.30.5000</t>
+          <t>9903.82.09,8302.42.3065</t>
         </is>
       </c>
       <c r="J855" t="inlineStr">
@@ -72026,7 +72026,7 @@
       </c>
       <c r="G856" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H856" t="inlineStr">
@@ -72036,7 +72036,7 @@
       </c>
       <c r="I856" t="inlineStr">
         <is>
-          <t>9903.82.09,8302.42.3065</t>
+          <t>9903.82.09,9403.99.9045</t>
         </is>
       </c>
       <c r="J856" t="inlineStr">
@@ -72109,7 +72109,7 @@
       </c>
       <c r="G857" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H857" t="inlineStr">
@@ -72119,7 +72119,7 @@
       </c>
       <c r="I857" t="inlineStr">
         <is>
-          <t>9903.82.09,9403.99.9045</t>
+          <t>9903.76.22,9403.40.9060</t>
         </is>
       </c>
       <c r="J857" t="inlineStr">
@@ -72166,12 +72166,12 @@
     <row r="858">
       <c r="A858" t="inlineStr">
         <is>
-          <t>4539589</t>
+          <t>4539623</t>
         </is>
       </c>
       <c r="B858" t="inlineStr">
         <is>
-          <t>EF4-0232907-4</t>
+          <t>EF4-0233010-6</t>
         </is>
       </c>
       <c r="C858" t="inlineStr">
@@ -72182,42 +72182,42 @@
       <c r="D858" t="inlineStr"/>
       <c r="E858" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="F858" t="inlineStr">
         <is>
-          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+          <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
       <c r="G858" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H858" t="inlineStr">
         <is>
-          <t>9903.03.06</t>
+          <t>9903.03.01</t>
         </is>
       </c>
       <c r="I858" t="inlineStr">
         <is>
-          <t>9903.76.22,9403.40.9060</t>
+          <t>9903.74.11,9903.94.06,8537.10.9170</t>
         </is>
       </c>
       <c r="J858" t="inlineStr">
         <is>
-          <t>NOLTE USA LLC</t>
+          <t>QUANTUM TECHNOLOGY SYSTEMS LLC</t>
         </is>
       </c>
       <c r="K858" t="inlineStr">
         <is>
-          <t>NOLUSA01</t>
+          <t>QUATEC01</t>
         </is>
       </c>
       <c r="L858" t="inlineStr">
         <is>
-          <t>46-224248300</t>
+          <t>33-167928800</t>
         </is>
       </c>
       <c r="M858" t="inlineStr">
@@ -72232,12 +72232,12 @@
       </c>
       <c r="O858" t="inlineStr">
         <is>
-          <t>NOLTE KUCHEN GMBH</t>
+          <t>ELCOM INTERNATIONAL PVT LTD</t>
         </is>
       </c>
       <c r="P858" t="inlineStr">
         <is>
-          <t>NOLTE KUCHEN GMBH</t>
+          <t>ELCOM INTERNATIONAL PVT LTD</t>
         </is>
       </c>
       <c r="Q858" t="inlineStr">
@@ -72249,83 +72249,3443 @@
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t>4539623</t>
+          <t>2565904</t>
         </is>
       </c>
       <c r="B859" t="inlineStr">
         <is>
-          <t>EF4-0233010-6</t>
+          <t>EF4-0231900-0</t>
         </is>
       </c>
       <c r="C859" t="inlineStr">
         <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>720204344</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F859" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I859" t="inlineStr">
+        <is>
+          <t>5603.14.9090</t>
+        </is>
+      </c>
+      <c r="J859" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K859" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L859" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M859" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N859" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O859" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P859" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q859" t="inlineStr">
+        <is>
+          <t>2026-05-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr"/>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F860" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I860" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J860" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K860" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L860" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M860" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N860" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O860" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P860" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q860" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr"/>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F861" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I861" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J861" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K861" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L861" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M861" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N861" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O861" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P861" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q861" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr"/>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F862" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I862" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J862" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K862" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L862" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M862" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N862" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O862" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P862" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q862" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr"/>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F863" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I863" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J863" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K863" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L863" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M863" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N863" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O863" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P863" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q863" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr"/>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F864" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I864" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J864" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K864" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L864" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M864" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N864" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O864" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P864" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q864" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr"/>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F865" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I865" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J865" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K865" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L865" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M865" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N865" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O865" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P865" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q865" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr"/>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F866" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I866" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J866" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K866" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L866" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M866" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N866" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O866" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P866" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q866" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2566069</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>EF4-0232118-8</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr"/>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F867" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I867" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J867" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K867" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L867" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M867" t="inlineStr">
+        <is>
+          <t>2026-07-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="N867" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O867" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P867" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q867" t="inlineStr">
+        <is>
+          <t>2026-05-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2566103</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>EF4-0232128-7</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>V8N81326921</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F868" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I868" t="inlineStr">
+        <is>
+          <t>8515.80.0080</t>
+        </is>
+      </c>
+      <c r="J868" t="inlineStr">
+        <is>
+          <t>VAUGHN BELTING CO INC</t>
+        </is>
+      </c>
+      <c r="K868" t="inlineStr">
+        <is>
+          <t>VAUBEL</t>
+        </is>
+      </c>
+      <c r="L868" t="inlineStr">
+        <is>
+          <t>58-166915900</t>
+        </is>
+      </c>
+      <c r="M868" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N868" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O868" t="inlineStr">
+        <is>
+          <t>ZEMAT TECHNOLOGY GROUP</t>
+        </is>
+      </c>
+      <c r="P868" t="inlineStr">
+        <is>
+          <t>ZEMAT TECHNOLOGY GROUP</t>
+        </is>
+      </c>
+      <c r="Q868" t="inlineStr">
+        <is>
+          <t>2026-05-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2566110</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>EF4-0232305-1</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>V8N81326921</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F869" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I869" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1061</t>
+        </is>
+      </c>
+      <c r="J869" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K869" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L869" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M869" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N869" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O869" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P869" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q869" t="inlineStr">
+        <is>
+          <t>2026-05-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2566190</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>EF4-0232316-8</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>V1626469798</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F870" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I870" t="inlineStr">
+        <is>
+          <t>1108.13.0010</t>
+        </is>
+      </c>
+      <c r="J870" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K870" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L870" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M870" t="inlineStr">
+        <is>
+          <t>2026-07-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="N870" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O870" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="P870" t="inlineStr">
+        <is>
+          <t>AKV LANGHOLT AMBA</t>
+        </is>
+      </c>
+      <c r="Q870" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2566250</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>EF4-0232498-4</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>V1626469798</t>
+        </is>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F871" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I871" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J871" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K871" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L871" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M871" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N871" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O871" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P871" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q871" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2566250</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>EF4-0232498-4</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>V1626469798</t>
+        </is>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F872" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I872" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J872" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K872" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L872" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M872" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N872" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O872" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P872" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q872" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2615770-8</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>EF4-0232512-2</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr"/>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F873" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I873" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J873" t="inlineStr">
+        <is>
+          <t>AUMUND CORPORATION</t>
+        </is>
+      </c>
+      <c r="K873" t="inlineStr">
+        <is>
+          <t>AUMCOR</t>
+        </is>
+      </c>
+      <c r="L873" t="inlineStr">
+        <is>
+          <t>58-138896800</t>
+        </is>
+      </c>
+      <c r="M873" t="inlineStr">
+        <is>
+          <t>2026-07-07 00:00:00</t>
+        </is>
+      </c>
+      <c r="N873" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O873" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="P873" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q873" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2566303</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>EF4-0232560-1</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr"/>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F874" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I874" t="inlineStr">
+        <is>
+          <t>1905.90.1050</t>
+        </is>
+      </c>
+      <c r="J874" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K874" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L874" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M874" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N874" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O874" t="inlineStr">
+        <is>
+          <t>HAFNER SEPTEUIL</t>
+        </is>
+      </c>
+      <c r="P874" t="inlineStr">
+        <is>
+          <t>HAFNER SEPTEUIL</t>
+        </is>
+      </c>
+      <c r="Q874" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2566303</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>EF4-0232560-1</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr"/>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F875" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I875" t="inlineStr">
+        <is>
+          <t>1905.90.1050</t>
+        </is>
+      </c>
+      <c r="J875" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K875" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L875" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M875" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N875" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O875" t="inlineStr">
+        <is>
+          <t>SMILDE BAKERY BV</t>
+        </is>
+      </c>
+      <c r="P875" t="inlineStr">
+        <is>
+          <t>SMILDE BAKERY BV</t>
+        </is>
+      </c>
+      <c r="Q875" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2566303</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>EF4-0232560-1</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr"/>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F876" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>1905.90.1050</t>
+        </is>
+      </c>
+      <c r="J876" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L876" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M876" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N876" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O876" t="inlineStr">
+        <is>
+          <t>HAFNER SEPTEUIL</t>
+        </is>
+      </c>
+      <c r="P876" t="inlineStr">
+        <is>
+          <t>HAFNER SEPTEUIL</t>
+        </is>
+      </c>
+      <c r="Q876" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2566304</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>EF4-0232561-9</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr"/>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F877" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I877" t="inlineStr">
+        <is>
+          <t>1905.90.1050</t>
+        </is>
+      </c>
+      <c r="J877" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K877" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L877" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M877" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N877" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O877" t="inlineStr">
+        <is>
+          <t>SMILDE BAKERY BV</t>
+        </is>
+      </c>
+      <c r="P877" t="inlineStr">
+        <is>
+          <t>SMILDE BAKERY BV</t>
+        </is>
+      </c>
+      <c r="Q877" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2566304</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>EF4-0232561-9</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr"/>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F878" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I878" t="inlineStr">
+        <is>
+          <t>1905.90.1050</t>
+        </is>
+      </c>
+      <c r="J878" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K878" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L878" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M878" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N878" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O878" t="inlineStr">
+        <is>
+          <t>HAFNER SEPTEUIL</t>
+        </is>
+      </c>
+      <c r="P878" t="inlineStr">
+        <is>
+          <t>HAFNER SEPTEUIL</t>
+        </is>
+      </c>
+      <c r="Q878" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2566304</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>EF4-0232561-9</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr"/>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F879" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G879" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H879" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I879" t="inlineStr">
+        <is>
+          <t>1905.90.1050</t>
+        </is>
+      </c>
+      <c r="J879" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K879" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L879" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M879" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N879" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O879" t="inlineStr">
+        <is>
+          <t>PIDY PRODUCTION-FRANCE</t>
+        </is>
+      </c>
+      <c r="P879" t="inlineStr">
+        <is>
+          <t>PIDY PRODUCTION-FRANCE</t>
+        </is>
+      </c>
+      <c r="Q879" t="inlineStr">
+        <is>
+          <t>2026-06-14 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>4539521</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>EF4-0232646-8</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
           <t>Air, Non-container</t>
         </is>
       </c>
-      <c r="D859" t="inlineStr"/>
-      <c r="E859" t="inlineStr">
-        <is>
-          <t>9903.03.01</t>
-        </is>
-      </c>
-      <c r="F859" t="inlineStr">
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>40654345771</t>
+        </is>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F880" t="inlineStr">
         <is>
           <t>SECTION 122 - 10% DUTY</t>
         </is>
       </c>
-      <c r="G859" t="inlineStr">
+      <c r="G880" t="inlineStr">
         <is>
           <t>001</t>
         </is>
       </c>
-      <c r="H859" t="inlineStr">
-        <is>
-          <t>9903.03.01</t>
-        </is>
-      </c>
-      <c r="I859" t="inlineStr">
-        <is>
-          <t>9903.74.11,9903.94.06,8537.10.9170</t>
-        </is>
-      </c>
-      <c r="J859" t="inlineStr">
-        <is>
-          <t>QUANTUM TECHNOLOGY SYSTEMS LLC</t>
-        </is>
-      </c>
-      <c r="K859" t="inlineStr">
-        <is>
-          <t>QUATEC01</t>
-        </is>
-      </c>
-      <c r="L859" t="inlineStr">
-        <is>
-          <t>33-167928800</t>
-        </is>
-      </c>
-      <c r="M859" t="inlineStr">
-        <is>
-          <t>2026-07-06 00:00:00</t>
-        </is>
-      </c>
-      <c r="N859" t="inlineStr">
-        <is>
-          <t>2026-07-07 00:00:00</t>
-        </is>
-      </c>
-      <c r="O859" t="inlineStr">
-        <is>
-          <t>ELCOM INTERNATIONAL PVT LTD</t>
-        </is>
-      </c>
-      <c r="P859" t="inlineStr">
-        <is>
-          <t>ELCOM INTERNATIONAL PVT LTD</t>
-        </is>
-      </c>
-      <c r="Q859" t="inlineStr">
-        <is>
-          <t>2026-07-06 00:00:00</t>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I880" t="inlineStr">
+        <is>
+          <t>8422.30.9120</t>
+        </is>
+      </c>
+      <c r="J880" t="inlineStr">
+        <is>
+          <t>HERMA US INC</t>
+        </is>
+      </c>
+      <c r="K880" t="inlineStr">
+        <is>
+          <t>HERUS01</t>
+        </is>
+      </c>
+      <c r="L880" t="inlineStr">
+        <is>
+          <t>61-178066000</t>
+        </is>
+      </c>
+      <c r="M880" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+      <c r="N880" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O880" t="inlineStr">
+        <is>
+          <t>HERMA UK LTD</t>
+        </is>
+      </c>
+      <c r="P880" t="inlineStr">
+        <is>
+          <t>HERMA UK LTD</t>
+        </is>
+      </c>
+      <c r="Q880" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2566348</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>EF4-0232730-0</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>40654345771</t>
+        </is>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F881" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H881" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I881" t="inlineStr">
+        <is>
+          <t>3926.90.9989</t>
+        </is>
+      </c>
+      <c r="J881" t="inlineStr">
+        <is>
+          <t>CON-PEARL AUTOMOTIVE INC</t>
+        </is>
+      </c>
+      <c r="K881" t="inlineStr">
+        <is>
+          <t>CONAUT04</t>
+        </is>
+      </c>
+      <c r="L881" t="inlineStr">
+        <is>
+          <t>82-412008100</t>
+        </is>
+      </c>
+      <c r="M881" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N881" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O881" t="inlineStr">
+        <is>
+          <t>GREIN GMBH</t>
+        </is>
+      </c>
+      <c r="P881" t="inlineStr">
+        <is>
+          <t>GREIN GMBH</t>
+        </is>
+      </c>
+      <c r="Q881" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2566305</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>EF4-0232763-1</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>VVS14102018</t>
+        </is>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F882" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I882" t="inlineStr">
+        <is>
+          <t>7019.66.4096</t>
+        </is>
+      </c>
+      <c r="J882" t="inlineStr">
+        <is>
+          <t>KAST TECHNICAL TEXTILES LP</t>
+        </is>
+      </c>
+      <c r="K882" t="inlineStr">
+        <is>
+          <t>KASTEC01</t>
+        </is>
+      </c>
+      <c r="L882" t="inlineStr">
+        <is>
+          <t>84-488647400</t>
+        </is>
+      </c>
+      <c r="M882" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N882" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O882" t="inlineStr">
+        <is>
+          <t>TOLNATEXT FONALFELDOLGOZO ES MUSZAK</t>
+        </is>
+      </c>
+      <c r="P882" t="inlineStr">
+        <is>
+          <t>TOLNATEXT FONALFELDOLGOZO ES MUSZAKISZOVET-GYARTO BT.</t>
+        </is>
+      </c>
+      <c r="Q882" t="inlineStr">
+        <is>
+          <t>2026-06-19 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2566201</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>EF4-0232799-5</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>VVS14102018</t>
+        </is>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F883" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I883" t="inlineStr">
+        <is>
+          <t>1109.00.9020</t>
+        </is>
+      </c>
+      <c r="J883" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K883" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L883" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M883" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N883" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O883" t="inlineStr">
+        <is>
+          <t>CARGILL BARBY</t>
+        </is>
+      </c>
+      <c r="P883" t="inlineStr">
+        <is>
+          <t>CARGILL BARBY</t>
+        </is>
+      </c>
+      <c r="Q883" t="inlineStr">
+        <is>
+          <t>2026-06-11 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr"/>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F884" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I884" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J884" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K884" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L884" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M884" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N884" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O884" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P884" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q884" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr"/>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F885" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I885" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J885" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K885" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L885" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M885" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N885" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O885" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P885" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q885" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr"/>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F886" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I886" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J886" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K886" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L886" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M886" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N886" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O886" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P886" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q886" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr"/>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F887" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I887" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J887" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K887" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L887" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M887" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N887" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O887" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P887" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q887" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr"/>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F888" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I888" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J888" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K888" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L888" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M888" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N888" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O888" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P888" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q888" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr"/>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F889" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I889" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J889" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K889" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L889" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M889" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N889" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O889" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P889" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q889" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr"/>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F890" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I890" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J890" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K890" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L890" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M890" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N890" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O890" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P890" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q890" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr"/>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F891" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I891" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J891" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K891" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L891" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M891" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N891" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O891" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P891" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q891" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr"/>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F892" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I892" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J892" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K892" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L892" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M892" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N892" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O892" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P892" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q892" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr"/>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I893" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J893" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K893" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L893" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M893" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N893" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O893" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P893" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q893" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr"/>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I894" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J894" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K894" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L894" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M894" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N894" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O894" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P894" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q894" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr"/>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I895" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J895" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K895" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L895" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M895" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N895" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O895" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P895" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q895" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr"/>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I896" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K896" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L896" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M896" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N896" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O896" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P896" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q896" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr"/>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I897" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K897" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L897" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M897" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N897" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O897" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P897" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q897" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr"/>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I898" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K898" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L898" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M898" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N898" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O898" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P898" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q898" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr"/>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K899" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L899" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M899" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N899" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="O899" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P899" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q899" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Append trimika data — 28 new rows, 910 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q899"/>
+  <dimension ref="A1:Q911"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -74364,28 +74364,28 @@
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566174</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232432-3</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D884" t="inlineStr"/>
       <c r="E884" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.03</t>
         </is>
       </c>
       <c r="F884" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
         </is>
       </c>
       <c r="G884" t="inlineStr">
@@ -74395,69 +74395,69 @@
       </c>
       <c r="H884" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.03</t>
         </is>
       </c>
       <c r="I884" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>2930.90.9231</t>
         </is>
       </c>
       <c r="J884" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>CASTLE CHEMICALS LTD</t>
         </is>
       </c>
       <c r="K884" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>CASCHE01</t>
         </is>
       </c>
       <c r="L884" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>151704-07138</t>
         </is>
       </c>
       <c r="M884" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="N884" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O884" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
         </is>
       </c>
       <c r="P884" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>HUBEI JIANGHAN NEW MATERIALS CO LTD</t>
         </is>
       </c>
       <c r="Q884" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-05-22 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566447</t>
         </is>
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232927-2</t>
         </is>
       </c>
       <c r="C885" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D885" t="inlineStr"/>
@@ -74473,7 +74473,7 @@
       </c>
       <c r="G885" t="inlineStr">
         <is>
-          <t>002</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H885" t="inlineStr">
@@ -74483,64 +74483,64 @@
       </c>
       <c r="I885" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>8422.40.9170</t>
         </is>
       </c>
       <c r="J885" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>KOCH, LIMITED PARTNERSHIP</t>
         </is>
       </c>
       <c r="K885" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>KOCLTD</t>
         </is>
       </c>
       <c r="L885" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>58-170306600</t>
         </is>
       </c>
       <c r="M885" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-11 00:00:00</t>
         </is>
       </c>
       <c r="N885" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O885" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="P885" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="Q885" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-24 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="886">
       <c r="A886" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566447</t>
         </is>
       </c>
       <c r="B886" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232927-2</t>
         </is>
       </c>
       <c r="C886" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D886" t="inlineStr"/>
@@ -74556,7 +74556,7 @@
       </c>
       <c r="G886" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H886" t="inlineStr">
@@ -74566,64 +74566,64 @@
       </c>
       <c r="I886" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>3920.20.0055</t>
         </is>
       </c>
       <c r="J886" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>KOCH, LIMITED PARTNERSHIP</t>
         </is>
       </c>
       <c r="K886" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>KOCLTD</t>
         </is>
       </c>
       <c r="L886" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>58-170306600</t>
         </is>
       </c>
       <c r="M886" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-11 00:00:00</t>
         </is>
       </c>
       <c r="N886" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O886" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="P886" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="Q886" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-24 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="887">
       <c r="A887" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566447</t>
         </is>
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232927-2</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D887" t="inlineStr"/>
@@ -74639,7 +74639,7 @@
       </c>
       <c r="G887" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H887" t="inlineStr">
@@ -74649,64 +74649,64 @@
       </c>
       <c r="I887" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>8422.40.9170</t>
         </is>
       </c>
       <c r="J887" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>KOCH, LIMITED PARTNERSHIP</t>
         </is>
       </c>
       <c r="K887" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>KOCLTD</t>
         </is>
       </c>
       <c r="L887" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>58-170306600</t>
         </is>
       </c>
       <c r="M887" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-11 00:00:00</t>
         </is>
       </c>
       <c r="N887" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O887" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="P887" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="Q887" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-24 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566447</t>
         </is>
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232927-2</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D888" t="inlineStr"/>
@@ -74722,7 +74722,7 @@
       </c>
       <c r="G888" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H888" t="inlineStr">
@@ -74732,64 +74732,64 @@
       </c>
       <c r="I888" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>3920.20.0055</t>
         </is>
       </c>
       <c r="J888" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>KOCH, LIMITED PARTNERSHIP</t>
         </is>
       </c>
       <c r="K888" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>KOCLTD</t>
         </is>
       </c>
       <c r="L888" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>58-170306600</t>
         </is>
       </c>
       <c r="M888" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-11 00:00:00</t>
         </is>
       </c>
       <c r="N888" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O888" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="P888" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PLASTICBAND S.A.</t>
         </is>
       </c>
       <c r="Q888" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-24 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2615842</t>
         </is>
       </c>
       <c r="B889" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232934-8</t>
         </is>
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Non-container</t>
         </is>
       </c>
       <c r="D889" t="inlineStr"/>
@@ -74805,7 +74805,7 @@
       </c>
       <c r="G889" t="inlineStr">
         <is>
-          <t>006</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H889" t="inlineStr">
@@ -74815,462 +74815,462 @@
       </c>
       <c r="I889" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>8517.62.0090</t>
         </is>
       </c>
       <c r="J889" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>PACKWISE INC</t>
         </is>
       </c>
       <c r="K889" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>PACINC01</t>
         </is>
       </c>
       <c r="L889" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>30-142471800</t>
         </is>
       </c>
       <c r="M889" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-06 00:00:00</t>
         </is>
       </c>
       <c r="N889" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O889" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PACKWISE GMBH</t>
         </is>
       </c>
       <c r="P889" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>PACKWISE GMBH</t>
         </is>
       </c>
       <c r="Q889" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-17 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566481</t>
         </is>
       </c>
       <c r="B890" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232996-7</t>
         </is>
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D890" t="inlineStr"/>
       <c r="E890" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F890" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G890" t="inlineStr">
         <is>
-          <t>007</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H890" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I890" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J890" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K890" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L890" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M890" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-10 00:00:00</t>
         </is>
       </c>
       <c r="N890" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O890" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P890" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q890" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="891">
       <c r="A891" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566481</t>
         </is>
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232996-7</t>
         </is>
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D891" t="inlineStr"/>
       <c r="E891" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F891" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G891" t="inlineStr">
         <is>
-          <t>008</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H891" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I891" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J891" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K891" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L891" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M891" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-10 00:00:00</t>
         </is>
       </c>
       <c r="N891" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O891" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P891" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q891" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="892">
       <c r="A892" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566481</t>
         </is>
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232996-7</t>
         </is>
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D892" t="inlineStr"/>
       <c r="E892" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F892" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G892" t="inlineStr">
         <is>
-          <t>009</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H892" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I892" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J892" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K892" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L892" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M892" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-10 00:00:00</t>
         </is>
       </c>
       <c r="N892" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O892" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P892" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q892" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="893">
       <c r="A893" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566481</t>
         </is>
       </c>
       <c r="B893" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232996-7</t>
         </is>
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D893" t="inlineStr"/>
       <c r="E893" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F893" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G893" t="inlineStr">
         <is>
-          <t>010</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H893" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I893" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J893" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K893" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L893" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M893" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-10 00:00:00</t>
         </is>
       </c>
       <c r="N893" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O893" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P893" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q893" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-26 00:00:00</t>
         </is>
       </c>
     </row>
     <row r="894">
       <c r="A894" t="inlineStr">
         <is>
-          <t>4539624</t>
+          <t>2566481</t>
         </is>
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>EF4-0233019-7</t>
+          <t>EF4-0232996-7</t>
         </is>
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>Air, Non-container</t>
+          <t>Vessel, Container</t>
         </is>
       </c>
       <c r="D894" t="inlineStr"/>
       <c r="E894" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="F894" t="inlineStr">
         <is>
-          <t>SECTION 122 - 10% DUTY</t>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
         </is>
       </c>
       <c r="G894" t="inlineStr">
         <is>
-          <t>011</t>
+          <t>005</t>
         </is>
       </c>
       <c r="H894" t="inlineStr">
         <is>
-          <t>9903.03.01</t>
+          <t>9903.03.06</t>
         </is>
       </c>
       <c r="I894" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
         </is>
       </c>
       <c r="J894" t="inlineStr">
         <is>
-          <t>DOBLA USA MFG LLC</t>
+          <t>BORGERS USA CORP</t>
         </is>
       </c>
       <c r="K894" t="inlineStr">
         <is>
-          <t>DOBUSA</t>
+          <t>BORUSA</t>
         </is>
       </c>
       <c r="L894" t="inlineStr">
         <is>
-          <t>41-218954800</t>
+          <t>65-117296500</t>
         </is>
       </c>
       <c r="M894" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-10 00:00:00</t>
         </is>
       </c>
       <c r="N894" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O894" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="P894" t="inlineStr">
         <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
+          <t>AUTONEUM CZ S.R.O.</t>
         </is>
       </c>
       <c r="Q894" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-06-26 00:00:00</t>
         </is>
       </c>
     </row>
@@ -75303,7 +75303,7 @@
       </c>
       <c r="G895" t="inlineStr">
         <is>
-          <t>012</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H895" t="inlineStr">
@@ -75313,7 +75313,7 @@
       </c>
       <c r="I895" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>1704.90.3590</t>
         </is>
       </c>
       <c r="J895" t="inlineStr">
@@ -75338,7 +75338,7 @@
       </c>
       <c r="N895" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O895" t="inlineStr">
@@ -75386,7 +75386,7 @@
       </c>
       <c r="G896" t="inlineStr">
         <is>
-          <t>013</t>
+          <t>002</t>
         </is>
       </c>
       <c r="H896" t="inlineStr">
@@ -75396,7 +75396,7 @@
       </c>
       <c r="I896" t="inlineStr">
         <is>
-          <t>1806.90.9085</t>
+          <t>1704.90.3590</t>
         </is>
       </c>
       <c r="J896" t="inlineStr">
@@ -75421,7 +75421,7 @@
       </c>
       <c r="N896" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O896" t="inlineStr">
@@ -75469,7 +75469,7 @@
       </c>
       <c r="G897" t="inlineStr">
         <is>
-          <t>014</t>
+          <t>003</t>
         </is>
       </c>
       <c r="H897" t="inlineStr">
@@ -75479,7 +75479,7 @@
       </c>
       <c r="I897" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>1806.90.9085</t>
         </is>
       </c>
       <c r="J897" t="inlineStr">
@@ -75504,7 +75504,7 @@
       </c>
       <c r="N897" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O897" t="inlineStr">
@@ -75552,7 +75552,7 @@
       </c>
       <c r="G898" t="inlineStr">
         <is>
-          <t>015</t>
+          <t>004</t>
         </is>
       </c>
       <c r="H898" t="inlineStr">
@@ -75562,7 +75562,7 @@
       </c>
       <c r="I898" t="inlineStr">
         <is>
-          <t>1704.90.3590</t>
+          <t>1806.90.9085</t>
         </is>
       </c>
       <c r="J898" t="inlineStr">
@@ -75587,7 +75587,7 @@
       </c>
       <c r="N898" t="inlineStr">
         <is>
-          <t>2026-07-08 00:00:00</t>
+          <t>2026-07-09 00:00:00</t>
         </is>
       </c>
       <c r="O898" t="inlineStr">
@@ -75635,55 +75635,1055 @@
       </c>
       <c r="G899" t="inlineStr">
         <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I899" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K899" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L899" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M899" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N899" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O899" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P899" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q899" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr"/>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I900" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J900" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K900" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L900" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M900" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N900" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O900" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P900" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q900" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr"/>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I901" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J901" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K901" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L901" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M901" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N901" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O901" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P901" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q901" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr"/>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I902" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J902" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K902" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L902" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M902" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N902" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O902" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P902" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q902" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr"/>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I903" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K903" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L903" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M903" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N903" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O903" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P903" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q903" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr"/>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I904" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L904" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M904" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N904" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O904" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P904" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q904" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr"/>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I905" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J905" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K905" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L905" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M905" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N905" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O905" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P905" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q905" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr"/>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I906" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J906" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K906" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L906" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M906" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N906" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O906" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P906" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q906" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr"/>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I907" t="inlineStr">
+        <is>
+          <t>1806.90.9085</t>
+        </is>
+      </c>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K907" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L907" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M907" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N907" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O907" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P907" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q907" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr"/>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I908" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J908" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K908" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L908" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M908" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N908" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O908" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P908" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q908" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr"/>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G909" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="H909" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I909" t="inlineStr">
+        <is>
+          <t>1704.90.3590</t>
+        </is>
+      </c>
+      <c r="J909" t="inlineStr">
+        <is>
+          <t>DOBLA USA MFG LLC</t>
+        </is>
+      </c>
+      <c r="K909" t="inlineStr">
+        <is>
+          <t>DOBUSA</t>
+        </is>
+      </c>
+      <c r="L909" t="inlineStr">
+        <is>
+          <t>41-218954800</t>
+        </is>
+      </c>
+      <c r="M909" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N909" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O909" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P909" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q909" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>4539624</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>EF4-0233019-7</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr"/>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
           <t>016</t>
         </is>
       </c>
-      <c r="H899" t="inlineStr">
-        <is>
-          <t>9903.03.01</t>
-        </is>
-      </c>
-      <c r="I899" t="inlineStr">
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I910" t="inlineStr">
         <is>
           <t>1806.90.9085</t>
         </is>
       </c>
-      <c r="J899" t="inlineStr">
+      <c r="J910" t="inlineStr">
         <is>
           <t>DOBLA USA MFG LLC</t>
         </is>
       </c>
-      <c r="K899" t="inlineStr">
+      <c r="K910" t="inlineStr">
         <is>
           <t>DOBUSA</t>
         </is>
       </c>
-      <c r="L899" t="inlineStr">
+      <c r="L910" t="inlineStr">
         <is>
           <t>41-218954800</t>
         </is>
       </c>
-      <c r="M899" t="inlineStr">
+      <c r="M910" t="inlineStr">
         <is>
           <t>2026-07-08 00:00:00</t>
         </is>
       </c>
-      <c r="N899" t="inlineStr">
+      <c r="N910" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O910" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="P910" t="inlineStr">
+        <is>
+          <t>DOBLA ASIA COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="Q910" t="inlineStr">
         <is>
           <t>2026-07-08 00:00:00</t>
         </is>
       </c>
-      <c r="O899" t="inlineStr">
-        <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="P899" t="inlineStr">
-        <is>
-          <t>DOBLA ASIA COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="Q899" t="inlineStr">
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>4539637</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>EF4-0233085-8</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>720204344</t>
+        </is>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I911" t="inlineStr">
+        <is>
+          <t>8438.90.9060</t>
+        </is>
+      </c>
+      <c r="J911" t="inlineStr">
+        <is>
+          <t>CANTRELL GAINCO GROUP INC</t>
+        </is>
+      </c>
+      <c r="K911" t="inlineStr">
+        <is>
+          <t>CANGAI01</t>
+        </is>
+      </c>
+      <c r="L911" t="inlineStr">
+        <is>
+          <t>31-151121700</t>
+        </is>
+      </c>
+      <c r="M911" t="inlineStr">
+        <is>
+          <t>2026-07-08 00:00:00</t>
+        </is>
+      </c>
+      <c r="N911" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="O911" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="P911" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="Q911" t="inlineStr">
         <is>
           <t>2026-07-08 00:00:00</t>
         </is>

</xml_diff>

<commit_message>
Append trimika data — 21 new rows, 1086 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1066"/>
+  <dimension ref="A1:Q1087"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -89606,6 +89606,1745 @@
         </is>
       </c>
     </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2566213</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>EF4-0232287-1</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr"/>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1067" t="inlineStr">
+        <is>
+          <t>5407.20.0000</t>
+        </is>
+      </c>
+      <c r="J1067" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K1067" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L1067" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M1067" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1067" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1067" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P1067" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q1067" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2566214</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>EF4-0232288-9</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr"/>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1068" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J1068" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K1068" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L1068" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M1068" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1068" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1068" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P1068" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q1068" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2566215</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>EF4-0232289-7</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>VA923894128</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1069" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J1069" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K1069" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L1069" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M1069" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1069" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1069" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P1069" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q1069" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2566083</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>EF4-0232468-7</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>VA923894128</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1070" t="inlineStr">
+        <is>
+          <t>3920.62.0090</t>
+        </is>
+      </c>
+      <c r="J1070" t="inlineStr">
+        <is>
+          <t>GULF ATLANTIC PACKAGING CORP</t>
+        </is>
+      </c>
+      <c r="K1070" t="inlineStr">
+        <is>
+          <t>GULATL</t>
+        </is>
+      </c>
+      <c r="L1070" t="inlineStr">
+        <is>
+          <t>58-184378700</t>
+        </is>
+      </c>
+      <c r="M1070" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1070" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1070" t="inlineStr">
+        <is>
+          <t>CONSENT FZCO</t>
+        </is>
+      </c>
+      <c r="P1070" t="inlineStr">
+        <is>
+          <t>CONSENT FZCO</t>
+        </is>
+      </c>
+      <c r="Q1070" t="inlineStr">
+        <is>
+          <t>2026-06-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>105504785</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>EF4-0232508-0</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr"/>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F1071" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G1071" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I1071" t="inlineStr"/>
+      <c r="J1071" t="inlineStr">
+        <is>
+          <t>DAVIS, SHANNON DENISE NICKENS</t>
+        </is>
+      </c>
+      <c r="K1071" t="inlineStr">
+        <is>
+          <t>DAVSHA02</t>
+        </is>
+      </c>
+      <c r="L1071" t="inlineStr"/>
+      <c r="M1071" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1071" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1071" t="inlineStr">
+        <is>
+          <t>MINI PLANT, BMW GROUP</t>
+        </is>
+      </c>
+      <c r="P1071" t="inlineStr">
+        <is>
+          <t>MINI PLANT, BMW GROUP</t>
+        </is>
+      </c>
+      <c r="Q1071" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>105504787</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>EF4-0232509-8</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr"/>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="F1072" t="inlineStr">
+        <is>
+          <t>EFFECTS US GOV EMP&amp;FAMLY/EVACU</t>
+        </is>
+      </c>
+      <c r="G1072" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>9805.00.50</t>
+        </is>
+      </c>
+      <c r="I1072" t="inlineStr"/>
+      <c r="J1072" t="inlineStr">
+        <is>
+          <t>RIVERA TORRES, HECTOR ANEWDY</t>
+        </is>
+      </c>
+      <c r="K1072" t="inlineStr">
+        <is>
+          <t>RIVTOR01</t>
+        </is>
+      </c>
+      <c r="L1072" t="inlineStr"/>
+      <c r="M1072" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1072" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1072" t="inlineStr">
+        <is>
+          <t>BMW AG</t>
+        </is>
+      </c>
+      <c r="P1072" t="inlineStr">
+        <is>
+          <t>BMW AG</t>
+        </is>
+      </c>
+      <c r="Q1072" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2566375</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>EF4-0232674-0</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr"/>
+      <c r="E1073" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1073" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1073" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1073" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1073" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J1073" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K1073" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L1073" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M1073" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1073" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1073" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P1073" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q1073" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2566375</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>EF4-0232674-0</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr"/>
+      <c r="E1074" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1074" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H1074" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1074" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J1074" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K1074" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L1074" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M1074" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1074" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1074" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P1074" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q1074" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2566375</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>EF4-0232674-0</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr"/>
+      <c r="E1075" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1075" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1075" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H1075" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1075" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J1075" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K1075" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L1075" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M1075" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1075" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1075" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P1075" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q1075" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2566375</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>EF4-0232674-0</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr"/>
+      <c r="E1076" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1076" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1076" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H1076" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1076" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J1076" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K1076" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L1076" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M1076" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1076" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1076" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P1076" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q1076" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2566375</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>EF4-0232674-0</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr"/>
+      <c r="E1077" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1077" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H1077" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1077" t="inlineStr">
+        <is>
+          <t>9903.74.11,9903.94.53,8708.29.5190</t>
+        </is>
+      </c>
+      <c r="J1077" t="inlineStr">
+        <is>
+          <t>HAGO AUTOMOTIVE CORP</t>
+        </is>
+      </c>
+      <c r="K1077" t="inlineStr">
+        <is>
+          <t>HAGAUT02</t>
+        </is>
+      </c>
+      <c r="L1077" t="inlineStr">
+        <is>
+          <t>47-447117700</t>
+        </is>
+      </c>
+      <c r="M1077" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1077" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1077" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="P1077" t="inlineStr">
+        <is>
+          <t>WALOR VOEHRENBACH GMBH</t>
+        </is>
+      </c>
+      <c r="Q1077" t="inlineStr">
+        <is>
+          <t>2026-06-17 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2566531</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>EF4-0232834-0</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr"/>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1078" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1078" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1078" t="inlineStr">
+        <is>
+          <t>8474.20.0010</t>
+        </is>
+      </c>
+      <c r="J1078" t="inlineStr">
+        <is>
+          <t>EDGE INNOVATE (NI) LTD</t>
+        </is>
+      </c>
+      <c r="K1078" t="inlineStr">
+        <is>
+          <t>EDGINN01</t>
+        </is>
+      </c>
+      <c r="L1078" t="inlineStr">
+        <is>
+          <t>135501-01432</t>
+        </is>
+      </c>
+      <c r="M1078" t="inlineStr">
+        <is>
+          <t>2026-07-09 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1078" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1078" t="inlineStr">
+        <is>
+          <t>EDGE INNOVATE (NI) LTD</t>
+        </is>
+      </c>
+      <c r="P1078" t="inlineStr">
+        <is>
+          <t>EDGE INNOVATE (NI) LTD</t>
+        </is>
+      </c>
+      <c r="Q1078" t="inlineStr">
+        <is>
+          <t>2026-06-25 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr"/>
+      <c r="E1079" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1079" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1079" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1079" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1079" t="inlineStr">
+        <is>
+          <t>3907.99.5050</t>
+        </is>
+      </c>
+      <c r="J1079" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1079" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1079" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1079" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1079" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1079" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1079" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1079" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr"/>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H1080" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1080" t="inlineStr">
+        <is>
+          <t>3909.20.0000</t>
+        </is>
+      </c>
+      <c r="J1080" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1080" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1080" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1080" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1080" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1080" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1080" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1080" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr"/>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H1081" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1081" t="inlineStr">
+        <is>
+          <t>3909.20.0000</t>
+        </is>
+      </c>
+      <c r="J1081" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1081" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1081" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1081" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1081" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1081" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1081" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1081" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr"/>
+      <c r="E1082" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1082" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H1082" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1082" t="inlineStr">
+        <is>
+          <t>3907.99.5050</t>
+        </is>
+      </c>
+      <c r="J1082" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1082" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1082" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1082" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1082" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1082" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1082" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1082" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr"/>
+      <c r="E1083" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1083" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H1083" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1083" t="inlineStr">
+        <is>
+          <t>2811.22.5000</t>
+        </is>
+      </c>
+      <c r="J1083" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1083" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1083" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1083" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1083" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1083" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1083" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1083" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr"/>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H1084" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1084" t="inlineStr">
+        <is>
+          <t>2909.43.0000</t>
+        </is>
+      </c>
+      <c r="J1084" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1084" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1084" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1084" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1084" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1084" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1084" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1084" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr"/>
+      <c r="E1085" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="F1085" t="inlineStr">
+        <is>
+          <t>S122 -EXCLUSION-EXEMPTED PRDTS</t>
+        </is>
+      </c>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H1085" t="inlineStr">
+        <is>
+          <t>9903.03.03</t>
+        </is>
+      </c>
+      <c r="I1085" t="inlineStr">
+        <is>
+          <t>2909.49.6000</t>
+        </is>
+      </c>
+      <c r="J1085" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1085" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1085" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1085" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1085" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1085" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1085" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1085" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2566559</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>EF4-0232876-1</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr"/>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H1086" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1086" t="inlineStr">
+        <is>
+          <t>3824.99.9397</t>
+        </is>
+      </c>
+      <c r="J1086" t="inlineStr">
+        <is>
+          <t>WEILBURGER NORTH AMERICA INC</t>
+        </is>
+      </c>
+      <c r="K1086" t="inlineStr">
+        <is>
+          <t>WEINOR03</t>
+        </is>
+      </c>
+      <c r="L1086" t="inlineStr">
+        <is>
+          <t>81-219562900</t>
+        </is>
+      </c>
+      <c r="M1086" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1086" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1086" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="P1086" t="inlineStr">
+        <is>
+          <t>WEILBURGER FRANCE</t>
+        </is>
+      </c>
+      <c r="Q1086" t="inlineStr">
+        <is>
+          <t>2026-06-23 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>4539663</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>EF4-0233148-4</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>721688801</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1087" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1087" t="inlineStr">
+        <is>
+          <t>8438.90.9060</t>
+        </is>
+      </c>
+      <c r="J1087" t="inlineStr">
+        <is>
+          <t>CANTRELL GAINCO GROUP INC</t>
+        </is>
+      </c>
+      <c r="K1087" t="inlineStr">
+        <is>
+          <t>CANGAI01</t>
+        </is>
+      </c>
+      <c r="L1087" t="inlineStr">
+        <is>
+          <t>31-151121700</t>
+        </is>
+      </c>
+      <c r="M1087" t="inlineStr">
+        <is>
+          <t>2026-07-10 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1087" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1087" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="P1087" t="inlineStr">
+        <is>
+          <t>O E CO LTD</t>
+        </is>
+      </c>
+      <c r="Q1087" t="inlineStr">
+        <is>
+          <t>2026-07-10 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Append trimika data — 34 new rows, 1148 total
</commit_message>
<xml_diff>
--- a/trimika_data.xlsx
+++ b/trimika_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1115"/>
+  <dimension ref="A1:Q1149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -93689,6 +93689,2860 @@
         </is>
       </c>
     </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2566125</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>EF4-0232324-2</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr"/>
+      <c r="E1116" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1116" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1116" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1116" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1116" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J1116" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K1116" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L1116" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M1116" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1116" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1116" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P1116" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q1116" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2566162</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>EF4-0232325-9</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr"/>
+      <c r="E1117" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1117" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1117" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>5903.90.3090</t>
+        </is>
+      </c>
+      <c r="J1117" t="inlineStr">
+        <is>
+          <t>VEER CORPORATIONS INC</t>
+        </is>
+      </c>
+      <c r="K1117" t="inlineStr">
+        <is>
+          <t>VEECOR01</t>
+        </is>
+      </c>
+      <c r="L1117" t="inlineStr">
+        <is>
+          <t>99-106989200</t>
+        </is>
+      </c>
+      <c r="M1117" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1117" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1117" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="P1117" t="inlineStr">
+        <is>
+          <t>VEER PLASTIC PVT LTD</t>
+        </is>
+      </c>
+      <c r="Q1117" t="inlineStr">
+        <is>
+          <t>2026-05-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2566200</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>EF4-0232352-3</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>V1626468857</t>
+        </is>
+      </c>
+      <c r="E1118" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1118" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1118" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1118" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1118" t="inlineStr">
+        <is>
+          <t>1109.00.1000</t>
+        </is>
+      </c>
+      <c r="J1118" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K1118" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L1118" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M1118" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1118" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1118" t="inlineStr">
+        <is>
+          <t>SEDAMYL UK</t>
+        </is>
+      </c>
+      <c r="P1118" t="inlineStr">
+        <is>
+          <t>SEDAMYL UK</t>
+        </is>
+      </c>
+      <c r="Q1118" t="inlineStr">
+        <is>
+          <t>2026-06-07 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2615764</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>EF4-0232403-4</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Vessel, Non-container</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>V1626468857</t>
+        </is>
+      </c>
+      <c r="E1119" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1119" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1119" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1119" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1119" t="inlineStr">
+        <is>
+          <t>9903.82.09,8483.10.5000</t>
+        </is>
+      </c>
+      <c r="J1119" t="inlineStr">
+        <is>
+          <t>AUMUND CORPORATION</t>
+        </is>
+      </c>
+      <c r="K1119" t="inlineStr">
+        <is>
+          <t>AUMCOR</t>
+        </is>
+      </c>
+      <c r="L1119" t="inlineStr">
+        <is>
+          <t>58-138896800</t>
+        </is>
+      </c>
+      <c r="M1119" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1119" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1119" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1119" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1119" t="inlineStr">
+        <is>
+          <t>2026-06-04 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2615765</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>EF4-0232407-5</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr"/>
+      <c r="E1120" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1120" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1120" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1120" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1120" t="inlineStr">
+        <is>
+          <t>9903.82.10,8431.39.0010</t>
+        </is>
+      </c>
+      <c r="J1120" t="inlineStr">
+        <is>
+          <t>AUMUND CORPORATION</t>
+        </is>
+      </c>
+      <c r="K1120" t="inlineStr">
+        <is>
+          <t>AUMCOR</t>
+        </is>
+      </c>
+      <c r="L1120" t="inlineStr">
+        <is>
+          <t>58-138896800</t>
+        </is>
+      </c>
+      <c r="M1120" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1120" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1120" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1120" t="inlineStr">
+        <is>
+          <t>AUMUND FOERDERTECHNIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1120" t="inlineStr">
+        <is>
+          <t>2026-06-08 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2566109</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>EF4-0232661-7</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr"/>
+      <c r="E1121" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1121" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1121" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1121" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1121" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1061</t>
+        </is>
+      </c>
+      <c r="J1121" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K1121" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L1121" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M1121" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1121" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1121" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P1121" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q1121" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2566224</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>EF4-0232663-3</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr"/>
+      <c r="E1122" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1122" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1122" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1122" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1122" t="inlineStr">
+        <is>
+          <t>9903.82.02,7223.00.1061</t>
+        </is>
+      </c>
+      <c r="J1122" t="inlineStr">
+        <is>
+          <t>VENUS WIRE INDUSTRIES PRIVATE LTD</t>
+        </is>
+      </c>
+      <c r="K1122" t="inlineStr">
+        <is>
+          <t>VENWIR</t>
+        </is>
+      </c>
+      <c r="L1122" t="inlineStr">
+        <is>
+          <t>993901-03595</t>
+        </is>
+      </c>
+      <c r="M1122" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1122" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1122" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="P1122" t="inlineStr">
+        <is>
+          <t>PRECISION METALS</t>
+        </is>
+      </c>
+      <c r="Q1122" t="inlineStr">
+        <is>
+          <t>2026-06-02 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2566488</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>EF4-0232805-0</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>V0710364576</t>
+        </is>
+      </c>
+      <c r="E1123" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1123" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1123" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1123" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1123" t="inlineStr">
+        <is>
+          <t>1109.00.9010</t>
+        </is>
+      </c>
+      <c r="J1123" t="inlineStr">
+        <is>
+          <t>ROYAL INGREDIENTS GROUP BV</t>
+        </is>
+      </c>
+      <c r="K1123" t="inlineStr">
+        <is>
+          <t>ROYINGRE</t>
+        </is>
+      </c>
+      <c r="L1123" t="inlineStr">
+        <is>
+          <t>074601-00962</t>
+        </is>
+      </c>
+      <c r="M1123" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1123" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1123" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="P1123" t="inlineStr">
+        <is>
+          <t>KROENER-STARKE BIO GMBH</t>
+        </is>
+      </c>
+      <c r="Q1123" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2566419</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>EF4-0232810-0</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>V0710364576</t>
+        </is>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1124" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1124" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1124" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1124" t="inlineStr">
+        <is>
+          <t>3921.90.5050</t>
+        </is>
+      </c>
+      <c r="J1124" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K1124" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L1124" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M1124" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1124" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1124" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P1124" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q1124" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2566419</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>EF4-0232810-0</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>V0710364576</t>
+        </is>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1125" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1125" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H1125" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1125" t="inlineStr">
+        <is>
+          <t>3921.90.5050</t>
+        </is>
+      </c>
+      <c r="J1125" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K1125" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L1125" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M1125" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1125" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1125" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P1125" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q1125" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2566419</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>EF4-0232810-0</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>V0710364576</t>
+        </is>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1126" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1126" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H1126" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1126" t="inlineStr">
+        <is>
+          <t>4811.59.4040</t>
+        </is>
+      </c>
+      <c r="J1126" t="inlineStr">
+        <is>
+          <t>BAUSCHLINNEMANN NORTH AMERICA</t>
+        </is>
+      </c>
+      <c r="K1126" t="inlineStr">
+        <is>
+          <t>BAULIN</t>
+        </is>
+      </c>
+      <c r="L1126" t="inlineStr">
+        <is>
+          <t>56-193913400</t>
+        </is>
+      </c>
+      <c r="M1126" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1126" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1126" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="P1126" t="inlineStr">
+        <is>
+          <t>SURTECO GMBH</t>
+        </is>
+      </c>
+      <c r="Q1126" t="inlineStr">
+        <is>
+          <t>2026-06-24 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2566122-1</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>EF4-0232869-6</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr"/>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1127" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1127" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1127" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1127" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0062</t>
+        </is>
+      </c>
+      <c r="J1127" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K1127" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L1127" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M1127" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1127" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1127" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P1127" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q1127" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2566122-2</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>EF4-0232871-2</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr"/>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="F1128" t="inlineStr">
+        <is>
+          <t>S122 EXCL,IRN/STL/ALUM,DERIV</t>
+        </is>
+      </c>
+      <c r="G1128" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1128" t="inlineStr">
+        <is>
+          <t>9903.03.06</t>
+        </is>
+      </c>
+      <c r="I1128" t="inlineStr">
+        <is>
+          <t>9903.82.02,7222.20.0062</t>
+        </is>
+      </c>
+      <c r="J1128" t="inlineStr">
+        <is>
+          <t>MESHA STEELS  LLC</t>
+        </is>
+      </c>
+      <c r="K1128" t="inlineStr">
+        <is>
+          <t>MESSTE</t>
+        </is>
+      </c>
+      <c r="L1128" t="inlineStr">
+        <is>
+          <t>20-274801900</t>
+        </is>
+      </c>
+      <c r="M1128" t="inlineStr">
+        <is>
+          <t>2026-07-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1128" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1128" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="P1128" t="inlineStr">
+        <is>
+          <t>BHANSALI BRIGHT BARS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="Q1128" t="inlineStr">
+        <is>
+          <t>2026-06-01 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr"/>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1129" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1129" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1129" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1129" t="inlineStr">
+        <is>
+          <t>3214.10.0090</t>
+        </is>
+      </c>
+      <c r="J1129" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1129" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1129" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1129" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1129" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1129" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="P1129" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="Q1129" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr"/>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1130" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1130" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H1130" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1130" t="inlineStr">
+        <is>
+          <t>3209.10.0000</t>
+        </is>
+      </c>
+      <c r="J1130" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1130" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1130" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1130" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1130" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1130" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="P1130" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="Q1130" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr"/>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1131" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1131" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="H1131" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1131" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1131" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1131" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1131" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1131" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1131" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1131" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="P1131" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="Q1131" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr"/>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1132" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1132" t="inlineStr">
+        <is>
+          <t>004</t>
+        </is>
+      </c>
+      <c r="H1132" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1132" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1132" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1132" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1132" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1132" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1132" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1132" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="P1132" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="Q1132" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr"/>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1133" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1133" t="inlineStr">
+        <is>
+          <t>005</t>
+        </is>
+      </c>
+      <c r="H1133" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1133" t="inlineStr">
+        <is>
+          <t>3824.99.9397</t>
+        </is>
+      </c>
+      <c r="J1133" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1133" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1133" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1133" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1133" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1133" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="P1133" t="inlineStr">
+        <is>
+          <t>FINALIN GMBH</t>
+        </is>
+      </c>
+      <c r="Q1133" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr"/>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1134" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1134" t="inlineStr">
+        <is>
+          <t>006</t>
+        </is>
+      </c>
+      <c r="H1134" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1134" t="inlineStr">
+        <is>
+          <t>3209.10.0000</t>
+        </is>
+      </c>
+      <c r="J1134" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1134" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1134" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1134" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1134" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1134" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1134" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1134" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr"/>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1135" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1135" t="inlineStr">
+        <is>
+          <t>007</t>
+        </is>
+      </c>
+      <c r="H1135" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1135" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1135" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1135" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1135" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1135" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1135" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1135" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1135" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1135" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr"/>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1136" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1136" t="inlineStr">
+        <is>
+          <t>008</t>
+        </is>
+      </c>
+      <c r="H1136" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1136" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1136" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1136" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1136" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1136" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1136" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1136" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1136" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1136" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr"/>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1137" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1137" t="inlineStr">
+        <is>
+          <t>009</t>
+        </is>
+      </c>
+      <c r="H1137" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1137" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1137" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1137" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1137" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1137" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1137" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1137" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1137" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1137" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr"/>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1138" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1138" t="inlineStr">
+        <is>
+          <t>010</t>
+        </is>
+      </c>
+      <c r="H1138" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1138" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1138" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1138" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1138" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1138" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1138" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1138" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1138" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1138" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr"/>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1139" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1139" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1139" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1139" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1139" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1139" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1139" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1139" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr"/>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>3209.10.0000</t>
+        </is>
+      </c>
+      <c r="J1140" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1140" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1140" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1140" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1140" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1140" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1140" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1140" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr"/>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1141" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1141" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1141" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1141" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1141" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1141" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1141" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1141" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr"/>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1142" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1142" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1142" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1142" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1142" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1142" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1142" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1142" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr"/>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1143" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1143" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1143" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1143" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1143" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1143" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1143" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1143" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr"/>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1144" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1144" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1144" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1144" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1144" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1144" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1144" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1144" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr"/>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1145" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1145" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1145" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1145" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1145" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1145" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1145" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1145" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr"/>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1146" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1146" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1146" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1146" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1146" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1146" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1146" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1146" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2566685</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>EF4-0233034-6</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Vessel, Container</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr"/>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>3209.90.0000</t>
+        </is>
+      </c>
+      <c r="J1147" t="inlineStr">
+        <is>
+          <t>MANKIEWICZ COATINGS, LLC</t>
+        </is>
+      </c>
+      <c r="K1147" t="inlineStr">
+        <is>
+          <t>MANCOAT</t>
+        </is>
+      </c>
+      <c r="L1147" t="inlineStr">
+        <is>
+          <t>56-202308900</t>
+        </is>
+      </c>
+      <c r="M1147" t="inlineStr">
+        <is>
+          <t>2026-07-15 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1147" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1147" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="P1147" t="inlineStr">
+        <is>
+          <t>NORIX LACKFABRIK GMBH</t>
+        </is>
+      </c>
+      <c r="Q1147" t="inlineStr">
+        <is>
+          <t>2026-07-05 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>4539641</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>EF4-0233087-4</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>01604345191</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>SECTION 122 - 10% DUTY</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>9903.03.01</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>3809.91.0000</t>
+        </is>
+      </c>
+      <c r="J1148" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICALS USA INC</t>
+        </is>
+      </c>
+      <c r="K1148" t="inlineStr">
+        <is>
+          <t>TANCHE</t>
+        </is>
+      </c>
+      <c r="L1148" t="inlineStr">
+        <is>
+          <t>74-324234000</t>
+        </is>
+      </c>
+      <c r="M1148" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1148" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1148" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICAL BV</t>
+        </is>
+      </c>
+      <c r="P1148" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICAL BV</t>
+        </is>
+      </c>
+      <c r="Q1148" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>4539641</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>EF4-0233087-4</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Air, Non-container</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>01604345191</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>ARTICLE OF CHINA,US NTE 20(F)</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>002</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>9903.88.03</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>9903.03.01,3809.91.0000</t>
+        </is>
+      </c>
+      <c r="J1149" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICALS USA INC</t>
+        </is>
+      </c>
+      <c r="K1149" t="inlineStr">
+        <is>
+          <t>TANCHE</t>
+        </is>
+      </c>
+      <c r="L1149" t="inlineStr">
+        <is>
+          <t>74-324234000</t>
+        </is>
+      </c>
+      <c r="M1149" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+      <c r="N1149" t="inlineStr">
+        <is>
+          <t>2026-07-13 00:00:00</t>
+        </is>
+      </c>
+      <c r="O1149" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICAL BV</t>
+        </is>
+      </c>
+      <c r="P1149" t="inlineStr">
+        <is>
+          <t>TANATEX CHEMICAL BV</t>
+        </is>
+      </c>
+      <c r="Q1149" t="inlineStr">
+        <is>
+          <t>2026-07-12 00:00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>